<commit_message>
Approvers' backup tables: 2026 base switched to 8+4, DMP campaign register margins added
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TjyVtBMeKRjjZMJmWM6RZp
</commit_message>
<xml_diff>
--- a/BU2027_вопросы_согласующих_база.xlsx
+++ b/BU2027_вопросы_согласующих_база.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="196">
   <si>
     <t xml:space="preserve">1. Вознаграждения рекламным агентствам (РА): 2026 vs 2027, млн руб. без НДС</t>
   </si>
   <si>
-    <t xml:space="preserve">Источники: бюджетная модель AdTech 2027 (cons 16.10, лист «Потребности»); Master AT Sep v9 (листы «10 PL», «20 Data_ACT», «Расшифровка»)</t>
+    <t xml:space="preserve">2026 = 8+4: факт янв–авг (журнал факта и «Расшифровка» мастера) + прогноз сен–дек (Master File FP&amp;A AdTech August v.1, лист Total). 2027 — модель cons 16.10</t>
   </si>
   <si>
     <t xml:space="preserve">1.1 Сводно</t>
@@ -59,10 +59,10 @@
     <t xml:space="preserve">Колонка «BU'26» в листе «Потребности»</t>
   </si>
   <si>
-    <t xml:space="preserve">2026 — FC 9+3 Master Sep v9 (9 мес. факт + 3 мес. прогноз)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q4 — по бюджету (ревизия BU), см. 1.2</t>
+    <t xml:space="preserve">2026 — FC 8+4 (8 мес. факт + 4 мес. прогноз, мастер август)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сен–дек — прогноз мастера августа, см. 1.2</t>
   </si>
   <si>
     <t xml:space="preserve">2027 — BU (модель cons 16.10)</t>
@@ -71,10 +71,10 @@
     <t xml:space="preserve">Фиксированная сумма 66,25 млн/мес. в реестре потребностей</t>
   </si>
   <si>
-    <t xml:space="preserve">Расхождение: FC 2026 в модели (354) и в актуальном мастере (261) различаются на ~93 млн — в материалах использован FC из модели. Рекомендуем согласовать базу 2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.2 Как формируется 2026 (Master Sep v9): начисления по месяцам</t>
+    <t xml:space="preserve">FC 2026 в модели (354, выручка 10 323) и 8+4 по мастеру августа (332, выручка 10 531) различаются на ~22 млн по РА.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2 Как формируется 2026 (8+4): начисления по месяцам</t>
   </si>
   <si>
     <t xml:space="preserve">Статья (по журналу факта)</t>
@@ -131,25 +131,25 @@
     <t xml:space="preserve">Премии РА: Instore</t>
   </si>
   <si>
-    <t xml:space="preserve">Прогноз Q4 (по бюджету, ревизия BU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого 2026 FC 9+3</t>
+    <t xml:space="preserve">Прогноз сен–дек (мастер август)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого 2026 FC 8+4</t>
   </si>
   <si>
     <t xml:space="preserve">Начисления неравномерны: премии РА признаются по итогам периодов, поэтому помесячная динамика не отражает ставку.</t>
   </si>
   <si>
-    <t xml:space="preserve">1.3 База 2026: выручка, полученная через РА (факт 9 мес.), и эффективная ставка</t>
+    <t xml:space="preserve">1.3 База 2026: выручка, полученная через РА (факт 8 мес.), и эффективная ставка</t>
   </si>
   <si>
     <t xml:space="preserve">Инвентарь</t>
   </si>
   <si>
-    <t xml:space="preserve">Выручка через РА, 9М</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Премии РА, 9М</t>
+    <t xml:space="preserve">Выручка через РА, 8М</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Премии РА, 8М</t>
   </si>
   <si>
     <t xml:space="preserve">Эфф. ставка</t>
@@ -170,16 +170,16 @@
     <t xml:space="preserve">Прочее (сторно/выплаты прошлых периодов)</t>
   </si>
   <si>
-    <t xml:space="preserve">Сторно премий 2025 г. в Q1 2026 и авто-загрузка сентября</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого 9М</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Доля выручки через РА: 41% выручки AdTech 9М (без М+)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">«Выручка через РА» — строки «Расшифровки» с реальным направлением «(РА)». Ставка оценочная: начисления 9М / выручка через РА 9М.</t>
+    <t xml:space="preserve">Сторно премий 2025 г. в Q1 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого 8М</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля выручки через РА: 43% выручки AdTech 8М (без М+)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">«Выручка через РА» — строки «Расшифровки» с реальным направлением «(РА)». Ставка оценочная: начисления 8М / выручка через РА 8М.</t>
   </si>
   <si>
     <t xml:space="preserve">1.4 Как сформирован 2027 (модель cons 16.10)</t>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">Модель cons 16.10</t>
   </si>
   <si>
-    <t xml:space="preserve">Доля выручки через РА (как в 9М 2026)</t>
+    <t xml:space="preserve">Доля выручки через РА (как в 8М 2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Допущение для оценки</t>
@@ -218,19 +218,19 @@
     <t xml:space="preserve">Подразумеваемая ставка при 795 млн</t>
   </si>
   <si>
-    <t xml:space="preserve">Сравнить со ставкой 9М 2026 (п. 1.3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">РА 2027 при ставке 9М 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ставка 9М 2026: 4.9%</t>
+    <t xml:space="preserve">Сравнить со ставкой 8М 2026 (п. 1.3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">РА 2027 при ставке 8М 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ставка 8М 2026: 5.8%</t>
   </si>
   <si>
     <t xml:space="preserve">2. DMP + Online: выручка, закупка трафика и маржинальность, млн руб. без НДС</t>
   </si>
   <si>
-    <t xml:space="preserve">Источники: модель AdTech 2027 cons 16.10 (листы «DMP», «Summary», «Потребности»); Master AT Sep v9 («10 PL», «20 Data_ACT», «Расшифровка»)</t>
+    <t xml:space="preserve">2027 — модель cons 16.10. 2026 = 8+4: факт янв–авг (журнал факта, «Расшифровка», реестр кампаний DMP) + прогноз сен–дек (мастер август)</t>
   </si>
   <si>
     <t xml:space="preserve">2.1 BU 2027 по направлениям (план команды DMP)</t>
@@ -296,7 +296,7 @@
     <t xml:space="preserve">Итого</t>
   </si>
   <si>
-    <t xml:space="preserve">2.3 Маржинальность 2026: два источника дают разную картину</t>
+    <t xml:space="preserve">2.3 Маржинальность 2026: модель, P&amp;L 8+4 и реестр кампаний DMP</t>
   </si>
   <si>
     <t xml:space="preserve">Источник</t>
@@ -311,34 +311,40 @@
     <t xml:space="preserve">Закупка 2026 — «План команды DMP на 2026» (лист DMP, блок 3)</t>
   </si>
   <si>
-    <t xml:space="preserve">Master Sep v9: факт 9М 2026</t>
+    <t xml:space="preserve">Факт 8М 2026 (P&amp;L)</t>
   </si>
   <si>
     <t xml:space="preserve">После корректировки в авг.: 120,7 млн перенесены с DMP+Online на «Other»</t>
   </si>
   <si>
-    <t xml:space="preserve">Master Sep v9: факт 9М 2026 без корректировки авг.</t>
+    <t xml:space="preserve">Факт 8М 2026 без корректировки авг.</t>
   </si>
   <si>
     <t xml:space="preserve">Если корректировку 120,7 вернуть на DMP+Online</t>
   </si>
   <si>
-    <t xml:space="preserve">Master Sep v9: прогноз Q4 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Q4 — выручка по методу прогноза, маркетинг — по бюджету</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Master Sep v9: FC 9+3 2026</t>
+    <t xml:space="preserve">Прогноз сен–дек 2026 (мастер август)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FC 8+4 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Год, с учётом корректировки авг.</t>
   </si>
   <si>
-    <t xml:space="preserve">Вывод для ответа: «маржа ~48% в 2026» — это план команды DMP в модели; по факту и прогнозу мастера маржа ниже (см. 2.4–2.5). Нужна сверка с командой DMP: какие расходы относятся к закупке трафика.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.4 2026 по месяцам (Master Sep v9)</t>
+    <t xml:space="preserve">FC 8+4 2026 без корректировки авг.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Справочно: реестр кампаний команды DMP, янв–авг</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Только стоимость размещений за вычетом рибейта; см. 2.5а</t>
+  </si>
+  <si>
+    <t xml:space="preserve">«Маржа ~48% в 2026» — план команды DMP в модели. По P&amp;L 8+4 — 50% (36%, если вернуть корректировку авг.); по реестру кампаний — 66%. В P&amp;L, кроме закупки размещений, отражены ТВ, блогеры, наружная реклама и акции (см. 2.5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4 2026 по месяцам (8+4)</t>
   </si>
   <si>
     <t xml:space="preserve">Выручка DMP+Online</t>
@@ -353,16 +359,16 @@
     <t xml:space="preserve">Маржинальность, %</t>
   </si>
   <si>
-    <t xml:space="preserve">Окт–дек — прогноз. Помесячная маржа волатильна из-за момента признания выручки и закрывающих документов площадок.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.5 Состав расходов DMP+Online, факт 9М 2026 (журнал факта)</t>
+    <t xml:space="preserve">Сен–дек — прогноз. Помесячная маржа волатильна из-за момента признания выручки и закрывающих документов площадок.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.5 Состав расходов DMP+Online, факт 8М 2026 (журнал факта)</t>
   </si>
   <si>
     <t xml:space="preserve">Вид расхода</t>
   </si>
   <si>
-    <t xml:space="preserve">Сумма 9М</t>
+    <t xml:space="preserve">Сумма 8М</t>
   </si>
   <si>
     <t xml:space="preserve">Закупка трафика на внешних площадках</t>
@@ -371,9 +377,6 @@
     <t xml:space="preserve">Размещение рекламы на ТВ</t>
   </si>
   <si>
-    <t xml:space="preserve">Сентябрь (загрузка корп. P&amp;L, без детализации)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Размещение у блогеров (Getblogger)</t>
   </si>
   <si>
@@ -395,6 +398,72 @@
     <t xml:space="preserve">Корректировка авг. (перенос на «Other»)</t>
   </si>
   <si>
+    <t xml:space="preserve">2.5а Фактическая маржа 2026 по типам размещения — реестр кампаний команды DMP (янв–авг)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тип размещения</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стоимость размещения</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рибейт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стоимость за вычетом рибейта</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кампаний</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OLV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Баннеры</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пакеты ТВ + онлайн (онлайн-часть)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Telegram (пост + картинка)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Площадка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Яндекс</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ВК видео</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пакеты ТВ + онлайн</t>
+  </si>
+  <si>
+    <t xml:space="preserve">МТ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пакет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТГ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Авито</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Яндекс БОНУС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Озон</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Яндекс Бонус частично</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Источник — листы «DMP 2026» и «DMP 2026 ТВ+онлайн» мастера августа (кампании по месяцу запуска). Выручка реестра не равна выручке P&amp;L за 8М: разный момент признания.</t>
+  </si>
+  <si>
     <t xml:space="preserve">2.6 Выручка по форматам (модель)</t>
   </si>
   <si>
@@ -431,16 +500,16 @@
     <t xml:space="preserve">В модели выручка DMP+Online разнесена на форматы по факту 8М 2026 (с корректировкой) — структура одинакова в обоих годах. Маржинальность по форматам в модели не считается (она задаётся по продуктам, п. 2.1).</t>
   </si>
   <si>
-    <t xml:space="preserve">В «Расшифровке» мастера формат проставлен только для ~8% выручки DMP+Online 9М — фактическую разбивку по форматам из мастера получить нельзя.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.7 Выручка DMP+Online 9М 2026 по типу рекламодателя и источнику бюджета («Расшифровка»)</t>
+    <t xml:space="preserve">В «Расшифровке» мастера формат проставлен только для ~8% выручки DMP+Online 8М — фактическую разбивку по форматам из мастера получить нельзя.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.7 Выручка DMP+Online 8М 2026 по типу рекламодателя и источнику бюджета («Расшифровка»)</t>
   </si>
   <si>
     <t xml:space="preserve">Тип рекламодателя</t>
   </si>
   <si>
-    <t xml:space="preserve">Выручка 9М</t>
+    <t xml:space="preserve">Выручка 8М</t>
   </si>
   <si>
     <t xml:space="preserve">Поставщики</t>
@@ -458,70 +527,52 @@
     <t xml:space="preserve">AdTech_Реклама и продвижение</t>
   </si>
   <si>
+    <t xml:space="preserve">Прочие маркетинговые активности</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ДМП</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пакеты лояльности и кросс-форматные акции</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ТВ интеграция поставщиков</t>
+  </si>
+  <si>
     <t xml:space="preserve">E-Commerce_Adtech</t>
   </si>
   <si>
-    <t xml:space="preserve">Прочие маркетинговые активности</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ДМП</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Пакеты лояльности и кросс-форматные акции</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ТВ интеграция поставщиков</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Реклама Компенсация</t>
-  </si>
-  <si>
     <t xml:space="preserve">Журнал Мой Магнит</t>
   </si>
   <si>
-    <t xml:space="preserve">Доп маржа Q3</t>
+    <t xml:space="preserve">Доп маржа Q1</t>
   </si>
   <si>
     <t xml:space="preserve">Регулярный оборотный бонус</t>
   </si>
   <si>
-    <t xml:space="preserve">Доп маржа Q1</t>
-  </si>
-  <si>
     <t xml:space="preserve">Доп маржа Q2</t>
   </si>
   <si>
     <t xml:space="preserve">Календаризация КУ, Q2</t>
   </si>
   <si>
-    <t xml:space="preserve">не указано</t>
-  </si>
-  <si>
     <t xml:space="preserve">Информационные услуги</t>
   </si>
   <si>
-    <t xml:space="preserve">Реклама и мероприятия в магазинах. BTL Мероприятия в магазинах</t>
-  </si>
-  <si>
     <t xml:space="preserve">E-Commerce_Реклама и продвижение (условное)</t>
   </si>
   <si>
-    <t xml:space="preserve">Прочие разовые условия</t>
-  </si>
-  <si>
     <t xml:space="preserve">Развитие ассортимента</t>
   </si>
   <si>
-    <t xml:space="preserve">Оплата каталога</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Все строки выручки DMP+Online в 2026 привязаны к КУ поставщиков (заполнен номер КУ). «Не РН AdTech, отражено в БиП» — 377 млн из 733: доход учтён в БиП по другим реальным направлениям.</t>
+    <t xml:space="preserve">Все строки выручки DMP+Online в 2026 привязаны к КУ поставщиков (заполнен номер КУ). Часть дохода учтена в БиП по другим реальным направлениям («Не РН AdTech»).</t>
   </si>
   <si>
     <t xml:space="preserve">Разбивки 2027 по типу рекламодателя и источнику бюджета в модели нет — план команды DMP задан по продуктам. Нужна от бизнеса.</t>
   </si>
   <si>
-    <t xml:space="preserve">2.8 Топ-10 рекламодателей DMP+Online, 9М 2026</t>
+    <t xml:space="preserve">2.8 Топ-10 рекламодателей DMP+Online, 8М 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Контрагент</t>
@@ -530,12 +581,12 @@
     <t xml:space="preserve">Тип</t>
   </si>
   <si>
+    <t xml:space="preserve">ЛАБ Индастриз ООО</t>
+  </si>
+  <si>
     <t xml:space="preserve">Рекитт Бенкизер ООО</t>
   </si>
   <si>
-    <t xml:space="preserve">ЛАБ Индастриз ООО</t>
-  </si>
-  <si>
     <t xml:space="preserve">Мондэлис Русь ООО (новый)</t>
   </si>
   <si>
@@ -545,29 +596,30 @@
     <t xml:space="preserve">Проктер энд Гэмбл Дистрибьюторская Компания ООО</t>
   </si>
   <si>
+    <t xml:space="preserve">Трейд-Сервис ООО</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ИнфоЛинк АО</t>
+  </si>
+  <si>
+    <t xml:space="preserve">МОРОЗКО ООО</t>
+  </si>
+  <si>
     <t xml:space="preserve">Нестле Россия ООО</t>
   </si>
   <si>
-    <t xml:space="preserve">Маревен Фуд Сэнтрал ООО</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ресурс ООО</t>
-  </si>
-  <si>
-    <t xml:space="preserve">МОРОЗКО ООО</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Аквалайн АО</t>
+    <t xml:space="preserve">Вимм-Билль-Данн АО (Московский филиал)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0;[RED]\-#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -669,7 +721,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -735,6 +787,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1003,7 +1063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1067,14 +1127,14 @@
         <v>12</v>
       </c>
       <c r="B8" s="7" t="n">
-        <v>261.074966560728</v>
+        <v>332.411346395055</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>10602.1840193036</v>
+        <v>10530.7067715848</v>
       </c>
       <c r="D8" s="8" t="n">
         <f aca="false">B8/C8</f>
-        <v>0.024624640176532</v>
+        <v>0.0315659103994811</v>
       </c>
       <c r="E8" s="9" t="s">
         <v>13</v>
@@ -1098,7 +1158,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>16</v>
       </c>
@@ -1183,12 +1243,9 @@
       <c r="I14" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J14" s="7" t="n">
-        <v>2.55310521</v>
-      </c>
       <c r="N14" s="7" t="n">
         <f aca="false">SUM(B14:M14)</f>
-        <v>-34.3098543</v>
+        <v>-36.86295951</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1219,9 +1276,6 @@
       <c r="I15" s="7" t="n">
         <v>0.939976</v>
       </c>
-      <c r="J15" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="N15" s="7" t="n">
         <f aca="false">SUM(B15:M15)</f>
         <v>94.60112079</v>
@@ -1255,9 +1309,6 @@
       <c r="I16" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="J16" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="N16" s="7" t="n">
         <f aca="false">SUM(B16:M16)</f>
         <v>4.75401409</v>
@@ -1291,9 +1342,6 @@
       <c r="I17" s="7" t="n">
         <v>1.17900459</v>
       </c>
-      <c r="J17" s="7" t="n">
-        <v>0</v>
-      </c>
       <c r="N17" s="7" t="n">
         <f aca="false">SUM(B17:M17)</f>
         <v>75.68845436</v>
@@ -1303,18 +1351,21 @@
       <c r="A18" s="3" t="s">
         <v>36</v>
       </c>
+      <c r="J18" s="7" t="n">
+        <v>43.8894850443278</v>
+      </c>
       <c r="K18" s="7" t="n">
-        <v>37.0923180264855</v>
+        <v>47.0923180264855</v>
       </c>
       <c r="L18" s="7" t="n">
-        <v>38.060136571781</v>
+        <v>48.060136571781</v>
       </c>
       <c r="M18" s="7" t="n">
-        <v>45.1887770224611</v>
+        <v>55.1887770224611</v>
       </c>
       <c r="N18" s="7" t="n">
         <f aca="false">SUM(B18:M18)</f>
-        <v>120.341231620728</v>
+        <v>194.230716665055</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1355,23 +1406,23 @@
       </c>
       <c r="J19" s="10" t="n">
         <f aca="false">SUM(J14:J18)</f>
-        <v>2.55310521</v>
+        <v>43.8894850443278</v>
       </c>
       <c r="K19" s="10" t="n">
         <f aca="false">SUM(K14:K18)</f>
-        <v>37.0923180264855</v>
+        <v>47.0923180264855</v>
       </c>
       <c r="L19" s="10" t="n">
         <f aca="false">SUM(L14:L18)</f>
-        <v>38.060136571781</v>
+        <v>48.060136571781</v>
       </c>
       <c r="M19" s="10" t="n">
         <f aca="false">SUM(M14:M18)</f>
-        <v>45.1887770224611</v>
+        <v>55.1887770224611</v>
       </c>
       <c r="N19" s="10" t="n">
         <f aca="false">SUM(N14:N18)</f>
-        <v>261.074966560728</v>
+        <v>332.411346395055</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1409,14 +1460,14 @@
         <v>44</v>
       </c>
       <c r="B24" s="7" t="n">
-        <v>847.26361341032</v>
+        <v>711.782499521939</v>
       </c>
       <c r="C24" s="7" t="n">
         <v>75.68845436</v>
       </c>
       <c r="D24" s="8" t="n">
         <f aca="false">IFERROR(C24/B24,"")</f>
-        <v>0.0893328276607401</v>
+        <v>0.10633649241283</v>
       </c>
       <c r="E24" s="9" t="s">
         <v>35</v>
@@ -1427,14 +1478,14 @@
         <v>45</v>
       </c>
       <c r="B25" s="7" t="n">
-        <v>221.070324877005</v>
+        <v>190.761574310513</v>
       </c>
       <c r="C25" s="7" t="n">
         <v>4.75401409</v>
       </c>
       <c r="D25" s="8" t="n">
         <f aca="false">IFERROR(C25/B25,"")</f>
-        <v>0.0215045329699721</v>
+        <v>0.0249212353545669</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>34</v>
@@ -1445,14 +1496,14 @@
         <v>46</v>
       </c>
       <c r="B26" s="7" t="n">
-        <v>1817.46908412241</v>
+        <v>1484.31679755366</v>
       </c>
       <c r="C26" s="7" t="n">
         <v>94.60112079</v>
       </c>
       <c r="D26" s="8" t="n">
         <f aca="false">IFERROR(C26/B26,"")</f>
-        <v>0.0520510206288761</v>
+        <v>0.0637337803802494</v>
       </c>
       <c r="E26" s="9" t="s">
         <v>47</v>
@@ -1463,7 +1514,7 @@
         <v>48</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>-34.3098543</v>
+        <v>-36.86295951</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>49</v>
@@ -1475,15 +1526,15 @@
       </c>
       <c r="B28" s="10" t="n">
         <f aca="false">SUM(B24:B27)</f>
-        <v>2885.80302240973</v>
+        <v>2386.86087138611</v>
       </c>
       <c r="C28" s="10" t="n">
         <f aca="false">SUM(C24:C27)</f>
-        <v>140.73373494</v>
+        <v>138.18062973</v>
       </c>
       <c r="D28" s="11" t="n">
         <f aca="false">IFERROR(C28/B28,"")</f>
-        <v>0.0487676164475298</v>
+        <v>0.0578922011695449</v>
       </c>
       <c r="E28" s="12" t="s">
         <v>51</v>
@@ -1631,7 +1682,7 @@
         <v>61</v>
       </c>
       <c r="B39" s="8" t="n">
-        <v>0.409489897135168</v>
+        <v>0.430091554994713</v>
       </c>
       <c r="C39" s="9" t="s">
         <v>62</v>
@@ -1643,7 +1694,7 @@
       </c>
       <c r="B40" s="7" t="n">
         <f aca="false">B38*B39</f>
-        <v>5964.72611492939</v>
+        <v>6264.81470687115</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1652,7 +1703,7 @@
       </c>
       <c r="B41" s="14" t="n">
         <f aca="false">795/B40</f>
-        <v>0.133283571564193</v>
+        <v>0.126899204078304</v>
       </c>
       <c r="C41" s="15" t="s">
         <v>65</v>
@@ -1663,8 +1714,8 @@
         <v>66</v>
       </c>
       <c r="B42" s="16" t="n">
-        <f aca="false">B40*0.0487676164475298</f>
-        <v>290.885475387441</v>
+        <f aca="false">B40*0.0578922011695449</f>
+        <v>362.683913300109</v>
       </c>
       <c r="C42" s="15" t="s">
         <v>67</v>
@@ -1686,7 +1737,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N101"/>
+  <dimension ref="A1:N117"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="54"/>
@@ -1932,18 +1983,18 @@
         <v>96</v>
       </c>
       <c r="B21" s="7" t="n">
-        <v>732.372564741753</v>
+        <v>530.702863852945</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>403.17353722</v>
+        <v>304.48541326</v>
       </c>
       <c r="D21" s="7" t="n">
         <f aca="false">B21-C21</f>
-        <v>329.199027521753</v>
+        <v>226.217450592945</v>
       </c>
       <c r="E21" s="8" t="n">
         <f aca="false">IFERROR(D21/B21,"")</f>
-        <v>0.449496667912232</v>
+        <v>0.426260090157773</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>97</v>
@@ -1954,18 +2005,18 @@
         <v>98</v>
       </c>
       <c r="B22" s="7" t="n">
-        <v>732.372564741753</v>
+        <v>530.702863852945</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>523.87353722</v>
+        <v>425.18541326</v>
       </c>
       <c r="D22" s="7" t="n">
         <f aca="false">B22-C22</f>
-        <v>208.499027521753</v>
+        <v>105.517450592945</v>
       </c>
       <c r="E22" s="8" t="n">
         <f aca="false">IFERROR(D22/B22,"")</f>
-        <v>0.28468983896915</v>
+        <v>0.198825854880224</v>
       </c>
       <c r="F22" s="9" t="s">
         <v>99</v>
@@ -1976,344 +2027,366 @@
         <v>100</v>
       </c>
       <c r="B23" s="7" t="n">
-        <v>329.017915993981</v>
+        <v>369.316632851684</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>283.639086031102</v>
+        <v>149.252797079744</v>
       </c>
       <c r="D23" s="7" t="n">
         <f aca="false">B23-C23</f>
-        <v>45.3788299628792</v>
+        <v>220.06383577194</v>
       </c>
       <c r="E23" s="8" t="n">
         <f aca="false">IFERROR(D23/B23,"")</f>
-        <v>0.13792206368394</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>101</v>
+        <v>0.595867654464176</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B24" s="10" t="n">
-        <v>1061.39048073574</v>
+        <v>900.019496704628</v>
       </c>
       <c r="C24" s="10" t="n">
-        <v>686.812623251102</v>
+        <v>453.738210339744</v>
       </c>
       <c r="D24" s="10" t="n">
         <f aca="false">B24-C24</f>
-        <v>374.577857484633</v>
+        <v>446.281286364885</v>
       </c>
       <c r="E24" s="11" t="n">
         <f aca="false">IFERROR(D24/B24,"")</f>
-        <v>0.352912395846045</v>
+        <v>0.495857354200569</v>
       </c>
       <c r="F24" s="12" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="B25" s="7" t="n">
+        <v>900.019496704628</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>574.438210339744</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <f aca="false">B25-C25</f>
+        <v>325.581286364885</v>
+      </c>
+      <c r="E25" s="8" t="n">
+        <f aca="false">IFERROR(D25/B25,"")</f>
+        <v>0.361749148276212</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="s">
+      <c r="B26" s="7" t="n">
+        <v>546.94153</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>186.683177653646</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <f aca="false">B26-C26</f>
+        <v>360.258352346354</v>
+      </c>
+      <c r="E26" s="8" t="n">
+        <f aca="false">IFERROR(D26/B26,"")</f>
+        <v>0.658677998626936</v>
+      </c>
+      <c r="F26" s="9" t="s">
         <v>105</v>
       </c>
     </row>
+    <row r="27" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B30" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C30" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D30" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E30" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="F30" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G28" s="6" t="s">
+      <c r="G30" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H28" s="6" t="s">
+      <c r="H30" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="I28" s="6" t="s">
+      <c r="I30" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="J28" s="6" t="s">
+      <c r="J30" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="K28" s="6" t="s">
+      <c r="K30" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="L28" s="6" t="s">
+      <c r="L30" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="M28" s="6" t="s">
+      <c r="M30" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="N28" s="6" t="s">
+      <c r="N30" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B29" s="7" t="n">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B31" s="7" t="n">
         <v>16.9387687250432</v>
       </c>
-      <c r="C29" s="7" t="n">
+      <c r="C31" s="7" t="n">
         <v>11.670591777213</v>
       </c>
-      <c r="D29" s="7" t="n">
+      <c r="D31" s="7" t="n">
         <v>3.3992407704918</v>
       </c>
-      <c r="E29" s="7" t="n">
+      <c r="E31" s="7" t="n">
         <v>25.4823725409836</v>
       </c>
-      <c r="F29" s="7" t="n">
+      <c r="F31" s="7" t="n">
         <v>57.6255045621643</v>
       </c>
-      <c r="G29" s="7" t="n">
+      <c r="G31" s="7" t="n">
         <v>213.320463671475</v>
       </c>
-      <c r="H29" s="7" t="n">
+      <c r="H31" s="7" t="n">
         <v>71.9327219331146</v>
       </c>
-      <c r="I29" s="7" t="n">
+      <c r="I31" s="7" t="n">
         <v>130.33319987246</v>
       </c>
-      <c r="J29" s="7" t="n">
-        <v>201.669700888808</v>
-      </c>
-      <c r="K29" s="7" t="n">
-        <v>91.8189533006459</v>
-      </c>
-      <c r="L29" s="7" t="n">
-        <v>107.122112184087</v>
-      </c>
-      <c r="M29" s="7" t="n">
-        <v>130.076850509248</v>
-      </c>
-      <c r="N29" s="7" t="n">
-        <f aca="false">SUM(B29:M29)</f>
-        <v>1061.39048073573</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B30" s="7" t="n">
-        <v>28.52889409</v>
-      </c>
-      <c r="C30" s="7" t="n">
-        <v>16.82913428</v>
-      </c>
-      <c r="D30" s="7" t="n">
-        <v>27.05948898</v>
-      </c>
-      <c r="E30" s="7" t="n">
-        <v>35.09782284</v>
-      </c>
-      <c r="F30" s="7" t="n">
-        <v>31.72780814</v>
-      </c>
-      <c r="G30" s="7" t="n">
-        <v>93.28901677</v>
-      </c>
-      <c r="H30" s="7" t="n">
-        <v>118.24761816</v>
-      </c>
-      <c r="I30" s="7" t="n">
-        <v>-46.29532942</v>
-      </c>
-      <c r="J30" s="7" t="n">
-        <v>98.68908338</v>
-      </c>
-      <c r="K30" s="7" t="n">
-        <v>95.9791790998034</v>
-      </c>
-      <c r="L30" s="7" t="n">
-        <v>86.6597652799349</v>
-      </c>
-      <c r="M30" s="7" t="n">
-        <v>101.000141651364</v>
-      </c>
-      <c r="N30" s="7" t="n">
-        <f aca="false">SUM(B30:M30)</f>
-        <v>686.812623251102</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="B31" s="10" t="n">
-        <f aca="false">B29-B30</f>
-        <v>-11.5901253649568</v>
-      </c>
-      <c r="C31" s="10" t="n">
-        <f aca="false">C29-C30</f>
-        <v>-5.158542502787</v>
-      </c>
-      <c r="D31" s="10" t="n">
-        <f aca="false">D29-D30</f>
-        <v>-23.6602482095082</v>
-      </c>
-      <c r="E31" s="10" t="n">
-        <f aca="false">E29-E30</f>
-        <v>-9.61545029901641</v>
-      </c>
-      <c r="F31" s="10" t="n">
-        <f aca="false">F29-F30</f>
-        <v>25.8976964221643</v>
-      </c>
-      <c r="G31" s="10" t="n">
-        <f aca="false">G29-G30</f>
-        <v>120.031446901475</v>
-      </c>
-      <c r="H31" s="10" t="n">
-        <f aca="false">H29-H30</f>
-        <v>-46.3148962268854</v>
-      </c>
-      <c r="I31" s="10" t="n">
-        <f aca="false">I29-I30</f>
-        <v>176.62852929246</v>
-      </c>
-      <c r="J31" s="10" t="n">
-        <f aca="false">J29-J30</f>
-        <v>102.980617508808</v>
-      </c>
-      <c r="K31" s="10" t="n">
-        <f aca="false">K29-K30</f>
-        <v>-4.16022579915746</v>
-      </c>
-      <c r="L31" s="10" t="n">
-        <f aca="false">L29-L30</f>
-        <v>20.462346904152</v>
-      </c>
-      <c r="M31" s="10" t="n">
-        <f aca="false">M29-M30</f>
-        <v>29.0767088578848</v>
-      </c>
-      <c r="N31" s="10" t="n">
-        <f aca="false">N29-N30</f>
-        <v>374.577857484633</v>
+      <c r="J31" s="7" t="n">
+        <v>75.205648644728</v>
+      </c>
+      <c r="K31" s="7" t="n">
+        <v>66.4565698783001</v>
+      </c>
+      <c r="L31" s="7" t="n">
+        <v>93.9568843826156</v>
+      </c>
+      <c r="M31" s="7" t="n">
+        <v>133.69752994604</v>
+      </c>
+      <c r="N31" s="7" t="n">
+        <f aca="false">SUM(B31:M31)</f>
+        <v>900.019496704628</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B32" s="8" t="n">
-        <f aca="false">IFERROR(B31/B29,"")</f>
-        <v>-0.684236590810838</v>
-      </c>
-      <c r="C32" s="8" t="n">
-        <f aca="false">IFERROR(C31/C29,"")</f>
-        <v>-0.442012076273556</v>
-      </c>
-      <c r="D32" s="8" t="n">
-        <f aca="false">IFERROR(D31/D29,"")</f>
+      <c r="B32" s="7" t="n">
+        <v>28.52889409</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>16.82913428</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>27.05948898</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>35.09782284</v>
+      </c>
+      <c r="F32" s="7" t="n">
+        <v>31.72780814</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>93.2890167700001</v>
+      </c>
+      <c r="H32" s="7" t="n">
+        <v>118.24857758</v>
+      </c>
+      <c r="I32" s="7" t="n">
+        <v>-46.29532942</v>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>37.602824322364</v>
+      </c>
+      <c r="K32" s="7" t="n">
+        <v>16.614142469575</v>
+      </c>
+      <c r="L32" s="7" t="n">
+        <v>28.1870653147847</v>
+      </c>
+      <c r="M32" s="7" t="n">
+        <v>66.84876497302</v>
+      </c>
+      <c r="N32" s="7" t="n">
+        <f aca="false">SUM(B32:M32)</f>
+        <v>453.738210339744</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B33" s="10" t="n">
+        <f aca="false">B31-B32</f>
+        <v>-11.5901253649569</v>
+      </c>
+      <c r="C33" s="10" t="n">
+        <f aca="false">C31-C32</f>
+        <v>-5.15854250278699</v>
+      </c>
+      <c r="D33" s="10" t="n">
+        <f aca="false">D31-D32</f>
+        <v>-23.6602482095082</v>
+      </c>
+      <c r="E33" s="10" t="n">
+        <f aca="false">E31-E32</f>
+        <v>-9.61545029901641</v>
+      </c>
+      <c r="F33" s="10" t="n">
+        <f aca="false">F31-F32</f>
+        <v>25.8976964221643</v>
+      </c>
+      <c r="G33" s="10" t="n">
+        <f aca="false">G31-G32</f>
+        <v>120.031446901475</v>
+      </c>
+      <c r="H33" s="10" t="n">
+        <f aca="false">H31-H32</f>
+        <v>-46.3158556468854</v>
+      </c>
+      <c r="I33" s="10" t="n">
+        <f aca="false">I31-I32</f>
+        <v>176.62852929246</v>
+      </c>
+      <c r="J33" s="10" t="n">
+        <f aca="false">J31-J32</f>
+        <v>37.602824322364</v>
+      </c>
+      <c r="K33" s="10" t="n">
+        <f aca="false">K31-K32</f>
+        <v>49.8424274087251</v>
+      </c>
+      <c r="L33" s="10" t="n">
+        <f aca="false">L31-L32</f>
+        <v>65.7698190678309</v>
+      </c>
+      <c r="M33" s="10" t="n">
+        <f aca="false">M31-M32</f>
+        <v>66.84876497302</v>
+      </c>
+      <c r="N33" s="10" t="n">
+        <f aca="false">N31-N32</f>
+        <v>446.281286364885</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="B34" s="8" t="n">
+        <f aca="false">IFERROR(B33/B31,"")</f>
+        <v>-0.684236590810843</v>
+      </c>
+      <c r="C34" s="8" t="n">
+        <f aca="false">IFERROR(C33/C31,"")</f>
+        <v>-0.442012076273554</v>
+      </c>
+      <c r="D34" s="8" t="n">
+        <f aca="false">IFERROR(D33/D31,"")</f>
         <v>-6.96045082034158</v>
       </c>
-      <c r="E32" s="8" t="n">
-        <f aca="false">IFERROR(E31/E29,"")</f>
+      <c r="E34" s="8" t="n">
+        <f aca="false">IFERROR(E33/E31,"")</f>
         <v>-0.377337325382547</v>
       </c>
-      <c r="F32" s="8" t="n">
-        <f aca="false">IFERROR(F31/F29,"")</f>
+      <c r="F34" s="8" t="n">
+        <f aca="false">IFERROR(F33/F31,"")</f>
         <v>0.449413790281468</v>
       </c>
-      <c r="G32" s="8" t="n">
-        <f aca="false">IFERROR(G31/G29,"")</f>
-        <v>0.562681351969729</v>
-      </c>
-      <c r="H32" s="8" t="n">
-        <f aca="false">IFERROR(H31/H29,"")</f>
-        <v>-0.643864085526341</v>
-      </c>
-      <c r="I32" s="8" t="n">
-        <f aca="false">IFERROR(I31/I29,"")</f>
+      <c r="G34" s="8" t="n">
+        <f aca="false">IFERROR(G33/G31,"")</f>
+        <v>0.562681351969728</v>
+      </c>
+      <c r="H34" s="8" t="n">
+        <f aca="false">IFERROR(H33/H31,"")</f>
+        <v>-0.643877423267138</v>
+      </c>
+      <c r="I34" s="8" t="n">
+        <f aca="false">IFERROR(I33/I31,"")</f>
         <v>1.35520749483097</v>
       </c>
-      <c r="J32" s="8" t="n">
-        <f aca="false">IFERROR(J31/J29,"")</f>
-        <v>0.510640007174836</v>
-      </c>
-      <c r="K32" s="8" t="n">
-        <f aca="false">IFERROR(K31/K29,"")</f>
-        <v>-0.045309009192639</v>
-      </c>
-      <c r="L32" s="8" t="n">
-        <f aca="false">IFERROR(L31/L29,"")</f>
-        <v>0.19101888944262</v>
-      </c>
-      <c r="M32" s="8" t="n">
-        <f aca="false">IFERROR(M31/M29,"")</f>
-        <v>0.223534846854379</v>
-      </c>
-      <c r="N32" s="8" t="n">
-        <f aca="false">IFERROR(N31/N29,"")</f>
-        <v>0.352912395846044</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3"/>
-    </row>
-    <row r="35" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
+      <c r="J34" s="8" t="n">
+        <f aca="false">IFERROR(J33/J31,"")</f>
+        <v>0.5</v>
+      </c>
+      <c r="K34" s="8" t="n">
+        <f aca="false">IFERROR(K33/K31,"")</f>
+        <v>0.75</v>
+      </c>
+      <c r="L34" s="8" t="n">
+        <f aca="false">IFERROR(L33/L31,"")</f>
+        <v>0.7</v>
+      </c>
+      <c r="M34" s="8" t="n">
+        <f aca="false">IFERROR(M33/M31,"")</f>
+        <v>0.5</v>
+      </c>
+      <c r="N34" s="8" t="n">
+        <f aca="false">IFERROR(N33/N31,"")</f>
+        <v>0.495857354200569</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="B36" s="6" t="s">
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3"/>
+    </row>
+    <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="4" t="s">
         <v>113</v>
       </c>
-      <c r="C36" s="6" t="s">
+    </row>
+    <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C38" s="6" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B37" s="7" t="n">
-        <v>282.49799362</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="B38" s="7" t="n">
-        <v>109.84879112</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2321,7 +2394,7 @@
         <v>116</v>
       </c>
       <c r="B39" s="7" t="n">
-        <v>98.68908338</v>
+        <v>282.49799362</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2329,7 +2402,7 @@
         <v>117</v>
       </c>
       <c r="B40" s="7" t="n">
-        <v>31.31843725</v>
+        <v>109.84879112</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2337,7 +2410,7 @@
         <v>118</v>
       </c>
       <c r="B41" s="7" t="n">
-        <v>19.726605</v>
+        <v>31.31843725</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2345,7 +2418,7 @@
         <v>119</v>
       </c>
       <c r="B42" s="7" t="n">
-        <v>16.0624436</v>
+        <v>19.726605</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2353,7 +2426,7 @@
         <v>120</v>
       </c>
       <c r="B43" s="7" t="n">
-        <v>9.92231206</v>
+        <v>16.0624436</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2361,7 +2434,7 @@
         <v>121</v>
       </c>
       <c r="B44" s="7" t="n">
-        <v>2.15214708</v>
+        <v>9.92231206</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2369,7 +2442,7 @@
         <v>122</v>
       </c>
       <c r="B45" s="7" t="n">
-        <v>-46.34583669</v>
+        <v>2.15214708</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2377,68 +2450,56 @@
         <v>123</v>
       </c>
       <c r="B46" s="7" t="n">
+        <v>-46.34583669</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B47" s="7" t="n">
         <v>-120.6984392</v>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="4" t="s">
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="B47" s="10" t="n">
-        <f aca="false">SUM(B37:B46)</f>
-        <v>403.17353722</v>
-      </c>
-      <c r="C47" s="12"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="3"/>
+      <c r="B48" s="10" t="n">
+        <f aca="false">SUM(B39:B47)</f>
+        <v>304.48445384</v>
+      </c>
+      <c r="C48" s="12"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="s">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B50" s="6" t="s">
+    </row>
+    <row r="51" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="B51" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C51" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="D51" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="E50" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="F50" s="6" t="s">
+      <c r="E51" s="6" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="3" t="s">
+      <c r="F51" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G51" s="6" t="s">
         <v>130</v>
-      </c>
-      <c r="B51" s="7" t="n">
-        <v>768.821180909195</v>
-      </c>
-      <c r="C51" s="8" t="n">
-        <f aca="false">B51/B$55</f>
-        <v>0.778947498388243</v>
-      </c>
-      <c r="D51" s="7" t="n">
-        <v>1246.31599742119</v>
-      </c>
-      <c r="E51" s="8" t="n">
-        <f aca="false">D51/D$55</f>
-        <v>0.778947498388243</v>
-      </c>
-      <c r="F51" s="7" t="n">
-        <f aca="false">D51-B51</f>
-        <v>477.494816511992</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2446,22 +2507,24 @@
         <v>131</v>
       </c>
       <c r="B52" s="7" t="n">
-        <v>192.791639187493</v>
-      </c>
-      <c r="C52" s="8" t="n">
-        <f aca="false">B52/B$55</f>
-        <v>0.195330941426032</v>
+        <v>267.84</v>
+      </c>
+      <c r="C52" s="7" t="n">
+        <v>122.937286453089</v>
       </c>
       <c r="D52" s="7" t="n">
-        <v>312.529506281651</v>
-      </c>
-      <c r="E52" s="8" t="n">
-        <f aca="false">D52/D$55</f>
-        <v>0.195330941426032</v>
-      </c>
-      <c r="F52" s="7" t="n">
-        <f aca="false">D52-B52</f>
-        <v>119.737867094157</v>
+        <v>26.3749593387</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <f aca="false">C52-D52</f>
+        <v>96.5623271143886</v>
+      </c>
+      <c r="F52" s="8" t="n">
+        <f aca="false">IFERROR(1-E52/B52,"")</f>
+        <v>0.639477572004224</v>
+      </c>
+      <c r="G52" s="17" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2469,22 +2532,24 @@
         <v>132</v>
       </c>
       <c r="B53" s="7" t="n">
-        <v>18.942306944518</v>
-      </c>
-      <c r="C53" s="8" t="n">
-        <f aca="false">B53/B$55</f>
-        <v>0.0191918003490557</v>
+        <v>149.76153</v>
+      </c>
+      <c r="C53" s="7" t="n">
+        <v>42.5467100504</v>
       </c>
       <c r="D53" s="7" t="n">
-        <v>30.7068805584891</v>
-      </c>
-      <c r="E53" s="8" t="n">
-        <f aca="false">D53/D$55</f>
-        <v>0.0191918003490557</v>
-      </c>
-      <c r="F53" s="7" t="n">
-        <f aca="false">D53-B53</f>
-        <v>11.7645736139711</v>
+        <v>6.25306026000001</v>
+      </c>
+      <c r="E53" s="7" t="n">
+        <f aca="false">C53-D53</f>
+        <v>36.2936497904</v>
+      </c>
+      <c r="F53" s="8" t="n">
+        <f aca="false">IFERROR(1-E53/B53,"")</f>
+        <v>0.75765705792135</v>
+      </c>
+      <c r="G53" s="17" t="n">
+        <v>157</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2492,574 +2557,941 @@
         <v>133</v>
       </c>
       <c r="B54" s="7" t="n">
-        <v>6.44487295879252</v>
-      </c>
-      <c r="C54" s="8" t="n">
-        <f aca="false">B54/B$55</f>
-        <v>0.00652975983666923</v>
+        <v>88</v>
+      </c>
+      <c r="C54" s="7" t="n">
+        <v>55.3283389957002</v>
       </c>
       <c r="D54" s="7" t="n">
-        <v>10.4476157386707</v>
-      </c>
-      <c r="E54" s="8" t="n">
-        <f aca="false">D54/D$55</f>
-        <v>0.00652975983666922</v>
-      </c>
-      <c r="F54" s="7" t="n">
-        <f aca="false">D54-B54</f>
-        <v>4.00274277987822</v>
+        <v>10.2444350668432</v>
+      </c>
+      <c r="E54" s="7" t="n">
+        <f aca="false">C54-D54</f>
+        <v>45.083903928857</v>
+      </c>
+      <c r="F54" s="8" t="n">
+        <f aca="false">IFERROR(1-E54/B54,"")</f>
+        <v>0.487682909899352</v>
+      </c>
+      <c r="G54" s="17" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="4" t="s">
+      <c r="A55" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B55" s="10" t="n">
-        <f aca="false">SUM(B51:B54)</f>
-        <v>986.999999999999</v>
-      </c>
-      <c r="C55" s="12"/>
-      <c r="D55" s="10" t="n">
-        <f aca="false">SUM(D51:D54)</f>
-        <v>1600</v>
-      </c>
-      <c r="E55" s="12"/>
-      <c r="F55" s="10" t="n">
-        <f aca="false">D55-B55</f>
-        <v>612.999999999998</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="2" t="s">
+      <c r="B55" s="7" t="n">
+        <v>41.34</v>
+      </c>
+      <c r="C55" s="7" t="n">
+        <v>10.23309832</v>
+      </c>
+      <c r="D55" s="7" t="n">
+        <v>1.4898015</v>
+      </c>
+      <c r="E55" s="7" t="n">
+        <f aca="false">C55-D55</f>
+        <v>8.74329682</v>
+      </c>
+      <c r="F55" s="8" t="n">
+        <f aca="false">IFERROR(1-E55/B55,"")</f>
+        <v>0.788502737784228</v>
+      </c>
+      <c r="G55" s="17" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B56" s="10" t="n">
+        <f aca="false">SUM(B52:B55)</f>
+        <v>546.94153</v>
+      </c>
+      <c r="C56" s="10" t="n">
+        <f aca="false">SUM(C52:C55)</f>
+        <v>231.045433819189</v>
+      </c>
+      <c r="D56" s="10" t="n">
+        <f aca="false">SUM(D52:D55)</f>
+        <v>44.3622561655432</v>
+      </c>
+      <c r="E56" s="10" t="n">
+        <f aca="false">C56-D56</f>
+        <v>186.683177653646</v>
+      </c>
+      <c r="F56" s="11" t="n">
+        <f aca="false">IFERROR(1-E56/B56,"")</f>
+        <v>0.658677998626936</v>
+      </c>
+      <c r="G56" s="18" t="n">
+        <f aca="false">SUM(G52:G55)</f>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3"/>
+    </row>
+    <row r="58" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="5" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="57" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="2" t="s">
+      <c r="B58" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="3" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="3"/>
-    </row>
-    <row r="59" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="4" t="s">
+      <c r="B59" s="7" t="n">
+        <v>130.8826</v>
+      </c>
+      <c r="C59" s="7" t="n">
+        <v>45.91374677</v>
+      </c>
+      <c r="D59" s="7" t="n">
+        <v>10.023402</v>
+      </c>
+      <c r="E59" s="7" t="n">
+        <f aca="false">C59-D59</f>
+        <v>35.89034477</v>
+      </c>
+      <c r="F59" s="8" t="n">
+        <f aca="false">IFERROR(1-E59/B59,"")</f>
+        <v>0.725782153089869</v>
+      </c>
+      <c r="G59" s="17" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="3" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="60" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="B60" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>127</v>
+      <c r="B60" s="7" t="n">
+        <v>117.71</v>
+      </c>
+      <c r="C60" s="7" t="n">
+        <v>38.3221292030885</v>
+      </c>
+      <c r="D60" s="7" t="n">
+        <v>9.1962275387</v>
+      </c>
+      <c r="E60" s="7" t="n">
+        <f aca="false">C60-D60</f>
+        <v>29.1259016643885</v>
+      </c>
+      <c r="F60" s="8" t="n">
+        <f aca="false">IFERROR(1-E60/B60,"")</f>
+        <v>0.752562215067636</v>
+      </c>
+      <c r="G60" s="17" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="B61" s="7" t="n">
-        <v>732.772564741752</v>
-      </c>
-      <c r="C61" s="8" t="n">
-        <f aca="false">B61/B$63</f>
-        <v>1.0005461701042</v>
+        <v>88</v>
+      </c>
+      <c r="C61" s="7" t="n">
+        <v>55.3283389957002</v>
+      </c>
+      <c r="D61" s="7" t="n">
+        <v>10.2444350668432</v>
+      </c>
+      <c r="E61" s="7" t="n">
+        <f aca="false">C61-D61</f>
+        <v>45.083903928857</v>
+      </c>
+      <c r="F61" s="8" t="n">
+        <f aca="false">IFERROR(1-E61/B61,"")</f>
+        <v>0.487682909899352</v>
+      </c>
+      <c r="G61" s="17" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B62" s="7" t="n">
+        <v>72.5556</v>
+      </c>
+      <c r="C62" s="7" t="n">
+        <v>33.69913131</v>
+      </c>
+      <c r="D62" s="7" t="n">
+        <v>5.567022</v>
+      </c>
+      <c r="E62" s="7" t="n">
+        <f aca="false">C62-D62</f>
+        <v>28.13210931</v>
+      </c>
+      <c r="F62" s="8" t="n">
+        <f aca="false">IFERROR(1-E62/B62,"")</f>
+        <v>0.612268256206275</v>
+      </c>
+      <c r="G62" s="17" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B63" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C63" s="7" t="n">
+        <v>34.94992511</v>
+      </c>
+      <c r="D63" s="7" t="n">
+        <v>7.2808718</v>
+      </c>
+      <c r="E63" s="7" t="n">
+        <f aca="false">C63-D63</f>
+        <v>27.66905331</v>
+      </c>
+      <c r="F63" s="8" t="n">
+        <f aca="false">IFERROR(1-E63/B63,"")</f>
+        <v>0.4466189338</v>
+      </c>
+      <c r="G63" s="17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="B62" s="7" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="C62" s="8" t="n">
-        <f aca="false">B62/B$63</f>
-        <v>-0.000546170104202425</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B63" s="10" t="n">
-        <f aca="false">SUM(B61:B62)</f>
-        <v>732.372564741752</v>
-      </c>
-      <c r="C63" s="12"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="3"/>
-    </row>
-    <row r="65" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="5" t="s">
+      <c r="B64" s="7" t="n">
+        <v>41.34</v>
+      </c>
+      <c r="C64" s="7" t="n">
+        <v>10.23309832</v>
+      </c>
+      <c r="D64" s="7" t="n">
+        <v>1.4898015</v>
+      </c>
+      <c r="E64" s="7" t="n">
+        <f aca="false">C64-D64</f>
+        <v>8.74329682</v>
+      </c>
+      <c r="F64" s="8" t="n">
+        <f aca="false">IFERROR(1-E64/B64,"")</f>
+        <v>0.788502737784228</v>
+      </c>
+      <c r="G64" s="17" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B65" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D65" s="6" t="s">
-        <v>127</v>
+      <c r="B65" s="7" t="n">
+        <v>23.50433</v>
+      </c>
+      <c r="C65" s="7" t="n">
+        <v>10.0834512204</v>
+      </c>
+      <c r="D65" s="7" t="n">
+        <v>0.4374</v>
+      </c>
+      <c r="E65" s="7" t="n">
+        <f aca="false">C65-D65</f>
+        <v>9.6460512204</v>
+      </c>
+      <c r="F65" s="8" t="n">
+        <f aca="false">IFERROR(1-E65/B65,"")</f>
+        <v>0.589605352698843</v>
+      </c>
+      <c r="G65" s="17" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B66" s="7" t="n">
-        <v>245.957262709098</v>
+        <v>12.359</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>74.8245547024533</v>
-      </c>
-      <c r="D66" s="8" t="n">
-        <f aca="false">B66/B$86</f>
-        <v>0.335836259507928</v>
+        <v>0.00033484</v>
+      </c>
+      <c r="D66" s="7" t="n">
+        <v>7.643E-005</v>
+      </c>
+      <c r="E66" s="7" t="n">
+        <f aca="false">C66-D66</f>
+        <v>0.00025841</v>
+      </c>
+      <c r="F66" s="8" t="n">
+        <f aca="false">IFERROR(1-E66/B66,"")</f>
+        <v>0.999979091350433</v>
+      </c>
+      <c r="G66" s="17" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B67" s="7" t="n">
-        <v>100.441894273966</v>
+        <v>6</v>
       </c>
       <c r="C67" s="7" t="n">
-        <v>6.10180348136066</v>
-      </c>
-      <c r="D67" s="8" t="n">
-        <f aca="false">B67/B$86</f>
-        <v>0.137145899654752</v>
+        <v>2.5152</v>
+      </c>
+      <c r="D67" s="7" t="n">
+        <v>0.123</v>
+      </c>
+      <c r="E67" s="7" t="n">
+        <f aca="false">C67-D67</f>
+        <v>2.3922</v>
+      </c>
+      <c r="F67" s="8" t="n">
+        <f aca="false">IFERROR(1-E67/B67,"")</f>
+        <v>0.6013</v>
+      </c>
+      <c r="G67" s="17" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B68" s="7" t="n">
+        <v>4.59</v>
+      </c>
+      <c r="C68" s="7" t="n">
+        <v>7.805E-005</v>
+      </c>
+      <c r="D68" s="7" t="n">
+        <v>1.983E-005</v>
+      </c>
+      <c r="E68" s="7" t="n">
+        <f aca="false">C68-D68</f>
+        <v>5.822E-005</v>
+      </c>
+      <c r="F68" s="8" t="n">
+        <f aca="false">IFERROR(1-E68/B68,"")</f>
+        <v>0.99998731590414</v>
+      </c>
+      <c r="G68" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="B68" s="7" t="n">
-        <v>95.0450792786885</v>
-      </c>
-      <c r="C68" s="7" t="n">
-        <v>19.9687522295081</v>
-      </c>
-      <c r="D68" s="8" t="n">
-        <f aca="false">B68/B$86</f>
-        <v>0.129776952133922</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="3" t="s">
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="3"/>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="B69" s="7" t="n">
-        <v>74.038</v>
-      </c>
-      <c r="C69" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D69" s="8" t="n">
-        <f aca="false">B69/B$86</f>
-        <v>0.101093355437348</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="3" t="s">
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="B70" s="7" t="n">
-        <v>63.91</v>
-      </c>
-      <c r="C70" s="7" t="n">
-        <v>61.02</v>
-      </c>
-      <c r="D70" s="8" t="n">
-        <f aca="false">B70/B$86</f>
-        <v>0.0872643283989424</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="3" t="s">
+      <c r="B72" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B71" s="7" t="n">
-        <v>60.85</v>
-      </c>
-      <c r="C71" s="7" t="n">
-        <v>12.85</v>
-      </c>
-      <c r="D71" s="8" t="n">
-        <f aca="false">B71/B$86</f>
-        <v>0.0830861271017939</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="3" t="s">
+      <c r="C72" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="B72" s="7" t="n">
-        <v>41.02</v>
-      </c>
-      <c r="C72" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D72" s="8" t="n">
-        <f aca="false">B72/B$86</f>
-        <v>0.0560097441859587</v>
+      <c r="D72" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B73" s="7" t="n">
-        <v>9.57</v>
-      </c>
-      <c r="C73" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D73" s="8" t="n">
-        <f aca="false">B73/B$86</f>
-        <v>0.013067119743043</v>
+        <v>768.821180909195</v>
+      </c>
+      <c r="C73" s="8" t="n">
+        <f aca="false">B73/B$77</f>
+        <v>0.778947498388243</v>
+      </c>
+      <c r="D73" s="7" t="n">
+        <v>1246.31599742119</v>
+      </c>
+      <c r="E73" s="8" t="n">
+        <f aca="false">D73/D$77</f>
+        <v>0.778947498388243</v>
+      </c>
+      <c r="F73" s="7" t="n">
+        <f aca="false">D73-B73</f>
+        <v>477.494816511992</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B74" s="7" t="n">
-        <v>7.71436192</v>
-      </c>
-      <c r="C74" s="7" t="n">
-        <v>3.07</v>
-      </c>
-      <c r="D74" s="8" t="n">
-        <f aca="false">B74/B$86</f>
-        <v>0.010533384634254</v>
+        <v>192.791639187493</v>
+      </c>
+      <c r="C74" s="8" t="n">
+        <f aca="false">B74/B$77</f>
+        <v>0.195330941426032</v>
+      </c>
+      <c r="D74" s="7" t="n">
+        <v>312.529506281651</v>
+      </c>
+      <c r="E74" s="8" t="n">
+        <f aca="false">D74/D$77</f>
+        <v>0.195330941426032</v>
+      </c>
+      <c r="F74" s="7" t="n">
+        <f aca="false">D74-B74</f>
+        <v>119.737867094157</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B75" s="7" t="n">
-        <v>7.11673</v>
-      </c>
-      <c r="C75" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D75" s="8" t="n">
-        <f aca="false">B75/B$86</f>
-        <v>0.0097173629142013</v>
+        <v>18.942306944518</v>
+      </c>
+      <c r="C75" s="8" t="n">
+        <f aca="false">B75/B$77</f>
+        <v>0.0191918003490557</v>
+      </c>
+      <c r="D75" s="7" t="n">
+        <v>30.7068805584891</v>
+      </c>
+      <c r="E75" s="8" t="n">
+        <f aca="false">D75/D$77</f>
+        <v>0.0191918003490557</v>
+      </c>
+      <c r="F75" s="7" t="n">
+        <f aca="false">D75-B75</f>
+        <v>11.7645736139711</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B76" s="7" t="n">
-        <v>6.35803083</v>
-      </c>
-      <c r="C76" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D76" s="8" t="n">
-        <f aca="false">B76/B$86</f>
-        <v>0.00868141590235832</v>
+        <v>6.44487295879252</v>
+      </c>
+      <c r="C76" s="8" t="n">
+        <f aca="false">B76/B$77</f>
+        <v>0.00652975983666923</v>
+      </c>
+      <c r="D76" s="7" t="n">
+        <v>10.4476157386707</v>
+      </c>
+      <c r="E76" s="8" t="n">
+        <f aca="false">D76/D$77</f>
+        <v>0.00652975983666922</v>
+      </c>
+      <c r="F76" s="7" t="n">
+        <f aca="false">D76-B76</f>
+        <v>4.00274277987822</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A77" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B77" s="7" t="n">
-        <v>5.06</v>
-      </c>
-      <c r="C77" s="7" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="D77" s="8" t="n">
-        <f aca="false">B77/B$86</f>
-        <v>0.00690905181816067</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A78" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="B78" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="C78" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D78" s="8" t="n">
-        <f aca="false">B78/B$86</f>
-        <v>0.00546170104202425</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="3" t="s">
+      <c r="A77" s="4" t="s">
         <v>157</v>
       </c>
-      <c r="B79" s="7" t="n">
-        <v>3.2112</v>
-      </c>
-      <c r="C79" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D79" s="8" t="n">
-        <f aca="false">B79/B$86</f>
-        <v>0.00438465359653706</v>
+      <c r="B77" s="10" t="n">
+        <f aca="false">SUM(B73:B76)</f>
+        <v>986.999999999999</v>
+      </c>
+      <c r="C77" s="12"/>
+      <c r="D77" s="10" t="n">
+        <f aca="false">SUM(D73:D76)</f>
+        <v>1600</v>
+      </c>
+      <c r="E77" s="12"/>
+      <c r="F77" s="10" t="n">
+        <f aca="false">D77-B77</f>
+        <v>612.999999999998</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="2" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="2" t="s">
+        <v>159</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="B80" s="7" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="C80" s="7" t="n">
-        <v>3.05</v>
-      </c>
-      <c r="D80" s="8" t="n">
-        <f aca="false">B80/B$86</f>
-        <v>0.00416454704454349</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A81" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="B81" s="7" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="C81" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D81" s="8" t="n">
-        <f aca="false">B81/B$86</f>
-        <v>0.00245776546891091</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A82" s="3" t="s">
+      <c r="A80" s="3"/>
+    </row>
+    <row r="81" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="4" t="s">
         <v>160</v>
       </c>
-      <c r="B82" s="7" t="n">
-        <v>1.19000573</v>
-      </c>
-      <c r="C82" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D82" s="8" t="n">
-        <f aca="false">B82/B$86</f>
-        <v>0.00162486388388896</v>
+    </row>
+    <row r="82" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B83" s="7" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="C83" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D83" s="8" t="n">
-        <f aca="false">B83/B$86</f>
-        <v>0.00139273376571618</v>
+        <v>531.102863852944</v>
+      </c>
+      <c r="C83" s="8" t="n">
+        <f aca="false">B83/B$85</f>
+        <v>1.00075371743257</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B84" s="7" t="n">
+        <v>-0.4</v>
+      </c>
+      <c r="C84" s="8" t="n">
+        <f aca="false">B84/B$85</f>
+        <v>-0.000753717432568516</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B85" s="10" t="n">
+        <f aca="false">SUM(B83:B84)</f>
+        <v>530.702863852945</v>
+      </c>
+      <c r="C85" s="12"/>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="3"/>
+    </row>
+    <row r="87" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B87" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="B84" s="7" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="C84" s="7" t="n">
+      <c r="C87" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D87" s="6" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B88" s="7" t="n">
+        <v>221.156488366715</v>
+      </c>
+      <c r="C88" s="7" t="n">
+        <v>66.1815752598303</v>
+      </c>
+      <c r="D88" s="8" t="n">
+        <f aca="false">B88/B$102</f>
+        <v>0.416723751519074</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B89" s="7" t="n">
+        <v>84.3864815491803</v>
+      </c>
+      <c r="C89" s="7" t="n">
+        <v>18.2999999999999</v>
+      </c>
+      <c r="D89" s="8" t="n">
+        <f aca="false">B89/B$102</f>
+        <v>0.159008905541846</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B90" s="7" t="n">
+        <v>74.038</v>
+      </c>
+      <c r="C90" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D84" s="8" t="n">
-        <f aca="false">B84/B$86</f>
-        <v>0.000696366882858091</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A85" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="B85" s="7" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="C85" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D85" s="8" t="n">
-        <f aca="false">B85/B$86</f>
-        <v>0.000696366882858091</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="B86" s="10" t="n">
-        <f aca="false">SUM(B66:B85)</f>
-        <v>732.372564741753</v>
-      </c>
-      <c r="C86" s="10" t="n">
-        <f aca="false">SUM(C66:C85)</f>
-        <v>181.395110413322</v>
-      </c>
-      <c r="D86" s="12"/>
-    </row>
-    <row r="87" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="2" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="2" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A89" s="3"/>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A90" s="4" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A91" s="5" t="s">
-        <v>167</v>
-      </c>
-      <c r="B91" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="C91" s="6" t="s">
-        <v>139</v>
+      <c r="D90" s="8" t="n">
+        <f aca="false">B90/B$102</f>
+        <v>0.139509328181269</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="B91" s="7" t="n">
+        <v>50.85</v>
+      </c>
+      <c r="C91" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D91" s="8" t="n">
+        <f aca="false">B91/B$102</f>
+        <v>0.0958163286152726</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="B92" s="9" t="s">
-        <v>140</v>
+        <v>171</v>
+      </c>
+      <c r="B92" s="7" t="n">
+        <v>40.85</v>
       </c>
       <c r="C92" s="7" t="n">
-        <v>84.7027480255559</v>
+        <v>12.85</v>
+      </c>
+      <c r="D92" s="8" t="n">
+        <f aca="false">B92/B$102</f>
+        <v>0.0769733928010597</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="B93" s="9" t="s">
-        <v>140</v>
+        <v>172</v>
+      </c>
+      <c r="B93" s="7" t="n">
+        <v>26.3338573770492</v>
       </c>
       <c r="C93" s="7" t="n">
-        <v>75.4599999999999</v>
+        <v>3.6273</v>
+      </c>
+      <c r="D93" s="8" t="n">
+        <f aca="false">B93/B$102</f>
+        <v>0.0496207184296374</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="B94" s="9" t="s">
-        <v>140</v>
+        <v>173</v>
+      </c>
+      <c r="B94" s="7" t="n">
+        <v>9.57</v>
       </c>
       <c r="C94" s="7" t="n">
-        <v>56.950821442623</v>
+        <v>0</v>
+      </c>
+      <c r="D94" s="8" t="n">
+        <f aca="false">B94/B$102</f>
+        <v>0.0180326895742017</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="B95" s="9" t="s">
-        <v>140</v>
+        <v>174</v>
+      </c>
+      <c r="B95" s="7" t="n">
+        <v>5.50803083</v>
       </c>
       <c r="C95" s="7" t="n">
-        <v>34.75</v>
+        <v>0</v>
+      </c>
+      <c r="D95" s="8" t="n">
+        <f aca="false">B95/B$102</f>
+        <v>0.0103787471392396</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="B96" s="9" t="s">
-        <v>140</v>
+        <v>175</v>
+      </c>
+      <c r="B96" s="7" t="n">
+        <v>5.2</v>
       </c>
       <c r="C96" s="7" t="n">
-        <v>34.246361</v>
+        <v>0</v>
+      </c>
+      <c r="D96" s="8" t="n">
+        <f aca="false">B96/B$102</f>
+        <v>0.00979832662339071</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B97" s="9" t="s">
-        <v>140</v>
+        <v>176</v>
+      </c>
+      <c r="B97" s="7" t="n">
+        <v>5.06</v>
       </c>
       <c r="C97" s="7" t="n">
-        <v>32.14</v>
+        <v>0.51</v>
+      </c>
+      <c r="D97" s="8" t="n">
+        <f aca="false">B97/B$102</f>
+        <v>0.00953452552199172</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="B98" s="9" t="s">
-        <v>140</v>
+        <v>177</v>
+      </c>
+      <c r="B98" s="7" t="n">
+        <v>4</v>
       </c>
       <c r="C98" s="7" t="n">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="D98" s="8" t="n">
+        <f aca="false">B98/B$102</f>
+        <v>0.00753717432568516</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="B99" s="9" t="s">
-        <v>140</v>
+        <v>178</v>
+      </c>
+      <c r="B99" s="7" t="n">
+        <v>2.05</v>
       </c>
       <c r="C99" s="7" t="n">
-        <v>28</v>
+        <v>2.05</v>
+      </c>
+      <c r="D99" s="8" t="n">
+        <f aca="false">B99/B$102</f>
+        <v>0.00386280184191364</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="B100" s="9" t="s">
-        <v>140</v>
+        <v>179</v>
+      </c>
+      <c r="B100" s="7" t="n">
+        <v>1.19000573</v>
       </c>
       <c r="C100" s="7" t="n">
-        <v>24.06022926</v>
+        <v>0</v>
+      </c>
+      <c r="D100" s="8" t="n">
+        <f aca="false">B100/B$102</f>
+        <v>0.00224232015889356</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="B101" s="9" t="s">
-        <v>140</v>
+        <v>180</v>
+      </c>
+      <c r="B101" s="7" t="n">
+        <v>0.51</v>
       </c>
       <c r="C101" s="7" t="n">
-        <v>24.00005</v>
+        <v>0</v>
+      </c>
+      <c r="D101" s="8" t="n">
+        <f aca="false">B101/B$102</f>
+        <v>0.000960989726524858</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A102" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B102" s="10" t="n">
+        <f aca="false">SUM(B88:B101)</f>
+        <v>530.702863852945</v>
+      </c>
+      <c r="C102" s="10" t="n">
+        <f aca="false">SUM(C88:C101)</f>
+        <v>153.51887525983</v>
+      </c>
+      <c r="D102" s="12"/>
+    </row>
+    <row r="103" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A103" s="2" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="2" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="3"/>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="B107" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="C107" s="6" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B108" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C108" s="7" t="n">
+        <v>61.0599999999998</v>
+      </c>
+    </row>
+    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A109" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B109" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C109" s="7" t="n">
+        <v>53.0435999999999</v>
+      </c>
+    </row>
+    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A110" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="B110" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C110" s="7" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A111" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B111" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C111" s="7" t="n">
+        <v>33.9</v>
+      </c>
+    </row>
+    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A112" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="B112" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C112" s="7" t="n">
+        <v>33.236361</v>
+      </c>
+    </row>
+    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A113" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="B113" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C113" s="7" t="n">
+        <v>25.3501545</v>
+      </c>
+    </row>
+    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A114" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B114" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C114" s="7" t="n">
+        <v>21.6000445</v>
+      </c>
+    </row>
+    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A115" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="B115" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C115" s="7" t="n">
+        <v>20.15022926</v>
+      </c>
+    </row>
+    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A116" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B116" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C116" s="7" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A117" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="B117" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="C117" s="7" t="n">
+        <v>14.15895</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agency fees sheet rebuilt on super-commission logic (base x average rate), reconciled with business wording
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TjyVtBMeKRjjZMJmWM6RZp
</commit_message>
<xml_diff>
--- a/BU2027_вопросы_согласующих_база.xlsx
+++ b/BU2027_вопросы_согласующих_база.xlsx
@@ -21,63 +21,159 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="196">
-  <si>
-    <t xml:space="preserve">1. Вознаграждения рекламным агентствам (РА): 2026 vs 2027, млн руб. без НДС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 = 8+4: факт янв–авг (журнал факта и «Расшифровка» мастера) + прогноз сен–дек (Master File FP&amp;A AdTech August v.1, лист Total). 2027 — модель cons 16.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.1 Сводно</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="200">
+  <si>
+    <t xml:space="preserve">1. Вознаграждения рекламным агентствам (суперкомиссия, СК): 2026 vs 2027, млн руб. без НДС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027 — модель cons 16.10 (лист «Потребности», блок «Вознаграждения рекламным агентствам 2027»). 2026 — BU 2026, FC в модели и 8+4 (мастер август).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.1 Расчёт 2027: база × средняя СК</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Группа бюджета</t>
+  </si>
+  <si>
+    <t xml:space="preserve">База (выручка)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Средняя СК</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выплаты РА</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Комментарий</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не поставщики</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В модели: 1,8 млрд × 30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Бренд-бюджеты (RMN, «Поставщики ММ»)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В модели: 0,85 млрд × 30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">795 млн — 66,25 млн/мес. в реестре потребностей</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.2 Сверка текстовки бизнеса с моделью (2027)</t>
   </si>
   <si>
     <t xml:space="preserve">Показатель</t>
   </si>
   <si>
-    <t xml:space="preserve">Сумма РА</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gross Revenue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Доля РА в выручке</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Комментарий</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 — FC в бюджетной модели (используется в материалах)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">База сравнения в презентации (FC 2026 из модели cons 10.09)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 — BU 2026 (реестр потребностей)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Колонка «BU'26» в листе «Потребности»</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026 — FC 8+4 (8 мес. факт + 4 мес. прогноз, мастер август)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сен–дек — прогноз мастера августа, см. 1.2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027 — BU (модель cons 16.10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фиксированная сумма 66,25 млн/мес. в реестре потребностей</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FC 2026 в модели (354, выручка 10 323) и 8+4 по мастеру августа (332, выручка 10 531) различаются на ~22 млн по РА.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.2 Как формируется 2026 (8+4): начисления по месяцам</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Статья (по журналу факта)</t>
+    <t xml:space="preserve">Текстовка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Модель</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разница</t>
+  </si>
+  <si>
+    <t xml:space="preserve">База: не поставщики</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В модели 1,8 млрд</t>
+  </si>
+  <si>
+    <t xml:space="preserve">База: бренд-бюджеты</t>
+  </si>
+  <si>
+    <t xml:space="preserve">База итого</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В модели 30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выплаты РА (база × СК)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">По текстовке получается 784, в бюджете 795</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Справочно: СК, при которой база 2,45 млрд даёт 795</t>
+  </si>
+  <si>
+    <t xml:space="preserve">32,4% — округляется до 32%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итог 795 сходится в обоих вариантах, но база и ставка в текстовке (2,45 млрд × 32%) отличаются от модели (2,65 млрд × 30%). Нужно выбрать один вариант: либо поправить текстовку под модель, либо обновить модель.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.3 Расчёт 2026: база × средняя СК</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BU 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FC в модели бюджета</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FC 8+4 (мастер август)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">База: внешние рекламодатели (не поставщики)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BU — 1,0 млрд; в 8+4 прогноз выручки от не поставщиков — 1,25 млрд</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Текстовка: 1 млрд × 36% = 360</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Текстовка опирается на BU 2026: база 1,0 млрд и СК ~35% (351,7 / 1 000). По 8+4 выручка от не поставщиков выше (1,25 млрд), а выплаты ниже (332), поэтому средняя СК — 26,7%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.4 Изменение средней СК 2027 к 2026, п.п.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вариант</t>
+  </si>
+  <si>
+    <t xml:space="preserve">СК 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">СК 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Изменение, п.п.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Текстовка (36% → 32%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Как в тексте бизнеса</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Модель: BU 2026 → BU 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35,2% → 30%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BU 2026 → текстовка 2027 (795 / 2,45 млрд)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">35,2% → 32,4%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Чтобы цифры и текст совпали, варианты формулировки: (а) по модели — «база 2,65 млрд × СК 30% = 795; в 2026 — 1,0 млрд × ~35% = 352; снижение средней СК ~5 п.п.»; (б) по текстовке — обновить в модели базу не поставщиков до 1,6 млрд и СК до 32,4%; снижение к BU 2026 — ~3 п.п.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.5 Помесячно: 2026 (8+4) и 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Статья 2026 (8+4)</t>
   </si>
   <si>
     <t xml:space="preserve">Янв</t>
@@ -137,267 +233,186 @@
     <t xml:space="preserve">Итого 2026 FC 8+4</t>
   </si>
   <si>
-    <t xml:space="preserve">Начисления неравномерны: премии РА признаются по итогам периодов, поэтому помесячная динамика не отражает ставку.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.3 База 2026: выручка, полученная через РА (факт 8 мес.), и эффективная ставка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Инвентарь</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Выручка через РА, 8М</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Премии РА, 8М</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Эфф. ставка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Digital Instore</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DMP / Online</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E-comm, пакеты, POSM, прочее</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Премии РА: AdTech; М+ (программа лояльности) исключена</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Прочее (сторно/выплаты прошлых периодов)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сторно премий 2025 г. в Q1 2026</t>
+    <t xml:space="preserve">Вознаграждения рекламным агентствам 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026: янв–авг — факт начислений (премии РА признаются по итогам периодов, помесячная динамика неравномерна); сен–дек — прогноз мастера августа. 2027 — 795 / 12.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. DMP + Online: выручка, закупка трафика и маржинальность, млн руб. без НДС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027 — модель cons 16.10. 2026 = 8+4: факт янв–авг (журнал факта, «Расшифровка», реестр кампаний DMP) + прогноз сен–дек (мастер август)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 BU 2027 по направлениям (план команды DMP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Направление</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржинальность</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закупка трафика</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Остаётся Магниту</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля выручки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пакеты и Онлайн+ТВ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Баннеры и OLV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Развитие новых площадок (SmartTV, Авито, МР)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого DMP + Online 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржинальность по направлениям — допущения плана команды DMP; закупка трафика = выручка × (1 − маржинальность).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 Закупка трафика 2027 по центрам ответственности (реестр потребностей)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Строка реестра</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сумма 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Комментарий в реестре</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMP+Online (Тарасов М., Кирилова А.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">«Суммы взяты из бюджета 2027 … рассчитаны от прогнозируемой выручки»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DMP+Online (ЦМ) (Ардаширов Д.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Комментария нет; в BU 2026 и факте 7М 2026 такой строки нет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3 Маржинальность 2026: модель, P&amp;L 8+4 и реестр кампаний DMP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Источник</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закупка трафика / маркетинг в интернете</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Модель cons 16.10: FC 2026 (база в презентации)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закупка 2026 — «План команды DMP на 2026» (лист DMP, блок 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Факт 8М 2026 (P&amp;L)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">После корректировки в авг.: 120,7 млн перенесены с DMP+Online на «Other»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Факт 8М 2026 без корректировки авг.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Если корректировку 120,7 вернуть на DMP+Online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прогноз сен–дек 2026 (мастер август)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FC 8+4 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Год, с учётом корректировки авг.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FC 8+4 2026 без корректировки авг.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Справочно: реестр кампаний команды DMP, янв–авг</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Только стоимость размещений за вычетом рибейта; см. 2.5а</t>
+  </si>
+  <si>
+    <t xml:space="preserve">«Маржа ~48% в 2026» — план команды DMP в модели. По P&amp;L 8+4 — 50% (36%, если вернуть корректировку авг.); по реестру кампаний — 66%. В P&amp;L, кроме закупки размещений, отражены ТВ, блогеры, наружная реклама и акции (см. 2.5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4 2026 по месяцам (8+4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка DMP+Online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маркетинг в интернете DMP+Online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржа</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржинальность, %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сен–дек — прогноз. Помесячная маржа волатильна из-за момента признания выручки и закрывающих документов площадок.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.5 Состав расходов DMP+Online, факт 8М 2026 (журнал факта)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вид расхода</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сумма 8М</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закупка трафика на внешних площадках</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Размещение рекламы на ТВ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Размещение у блогеров (Getblogger)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рекламные акции (лояльность)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Наружная реклама (растяжки, щиты, пиллары)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Размещение рекламы в интернете</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Агентские вознаграждения</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прочее (ЗНР, ОРД, без описания)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Корректировка авг. (перенос на «Other»)</t>
   </si>
   <si>
     <t xml:space="preserve">Итого 8М</t>
   </si>
   <si>
-    <t xml:space="preserve">Доля выручки через РА: 43% выручки AdTech 8М (без М+)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">«Выручка через РА» — строки «Расшифровки» с реальным направлением «(РА)». Ставка оценочная: начисления 8М / выручка через РА 8М.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.4 Как сформирован 2027 (модель cons 16.10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Статья</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вознаграждения рекламным агентствам</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Источник — реестр потребностей (ответственные: Мухутдинов Д., Соколов П.): фиксированная сумма 66,25 млн руб./мес. Ставка и база в модели не заданы — нужен расчёт от бизнеса.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.5 Справочно: что подразумевает 795 млн при структуре 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Значение</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gross Revenue 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Модель cons 16.10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Доля выручки через РА (как в 8М 2026)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Допущение для оценки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">База — выручка через РА 2027 (оценка)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Подразумеваемая ставка при 795 млн</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сравнить со ставкой 8М 2026 (п. 1.3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">РА 2027 при ставке 8М 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ставка 8М 2026: 5.8%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. DMP + Online: выручка, закупка трафика и маржинальность, млн руб. без НДС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027 — модель cons 16.10. 2026 = 8+4: факт янв–авг (журнал факта, «Расшифровка», реестр кампаний DMP) + прогноз сен–дек (мастер август)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.1 BU 2027 по направлениям (план команды DMP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Направление</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Выручка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маржинальность</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Закупка трафика</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Остаётся Магниту</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Доля выручки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Пакеты и Онлайн+ТВ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Баннеры и OLV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Развитие новых площадок (SmartTV, Авито, МР)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого DMP + Online 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маржинальность по направлениям — допущения плана команды DMP; закупка трафика = выручка × (1 − маржинальность).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2 Закупка трафика 2027 по центрам ответственности (реестр потребностей)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Строка реестра</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сумма 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Комментарий в реестре</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DMP+Online (Тарасов М., Кирилова А.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">«Суммы взяты из бюджета 2027 … рассчитаны от прогнозируемой выручки»</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DMP+Online (ЦМ) (Ардаширов Д.)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Комментария нет; в BU 2026 и факте 7М 2026 такой строки нет</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.3 Маржинальность 2026: модель, P&amp;L 8+4 и реестр кампаний DMP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Источник</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Закупка трафика / маркетинг в интернете</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Модель cons 16.10: FC 2026 (база в презентации)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Закупка 2026 — «План команды DMP на 2026» (лист DMP, блок 3)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Факт 8М 2026 (P&amp;L)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">После корректировки в авг.: 120,7 млн перенесены с DMP+Online на «Other»</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Факт 8М 2026 без корректировки авг.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Если корректировку 120,7 вернуть на DMP+Online</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Прогноз сен–дек 2026 (мастер август)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FC 8+4 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Год, с учётом корректировки авг.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FC 8+4 2026 без корректировки авг.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Справочно: реестр кампаний команды DMP, янв–авг</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Только стоимость размещений за вычетом рибейта; см. 2.5а</t>
-  </si>
-  <si>
-    <t xml:space="preserve">«Маржа ~48% в 2026» — план команды DMP в модели. По P&amp;L 8+4 — 50% (36%, если вернуть корректировку авг.); по реестру кампаний — 66%. В P&amp;L, кроме закупки размещений, отражены ТВ, блогеры, наружная реклама и акции (см. 2.5).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.4 2026 по месяцам (8+4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Выручка DMP+Online</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маркетинг в интернете DMP+Online</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маржа</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маржинальность, %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сен–дек — прогноз. Помесячная маржа волатильна из-за момента признания выручки и закрывающих документов площадок.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.5 Состав расходов DMP+Online, факт 8М 2026 (журнал факта)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вид расхода</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сумма 8М</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Закупка трафика на внешних площадках</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Размещение рекламы на ТВ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Размещение у блогеров (Getblogger)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Рекламные акции (лояльность)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Наружная реклама (растяжки, щиты, пиллары)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Размещение рекламы в интернете</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Агентские вознаграждения</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Прочее (ЗНР, ОРД, без описания)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Корректировка авг. (перенос на «Other»)</t>
-  </si>
-  <si>
     <t xml:space="preserve">2.5а Фактическая маржа 2026 по типам размещения — реестр кампаний команды DMP (янв–авг)</t>
   </si>
   <si>
@@ -513,9 +528,6 @@
   </si>
   <si>
     <t xml:space="preserve">Поставщики</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не поставщики</t>
   </si>
   <si>
     <t xml:space="preserve">Источник бюджета (реальное направление по КУ)</t>
@@ -615,11 +627,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0;[RED]\-#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -782,11 +795,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -794,7 +803,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1050,12 +1063,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="54"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1076,7 +1089,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
@@ -1093,19 +1106,19 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="7" t="n">
-        <v>354.4</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>10323.4492363</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <f aca="false">B6/C6</f>
-        <v>0.0343296113428674</v>
+        <v>1800</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D6" s="7" t="n">
+        <f aca="false">B6*C6</f>
+        <v>540</v>
       </c>
       <c r="E6" s="9" t="s">
         <v>9</v>
@@ -1116,609 +1129,670 @@
         <v>10</v>
       </c>
       <c r="B7" s="7" t="n">
-        <v>351.73</v>
+        <v>850</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <f aca="false">B7*C7</f>
+        <v>255</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="7" t="n">
-        <v>332.411346395055</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>10530.7067715848</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <f aca="false">B8/C8</f>
-        <v>0.0315659103994811</v>
-      </c>
-      <c r="E8" s="9" t="s">
+      <c r="B8" s="10" t="n">
+        <f aca="false">B6+B7</f>
+        <v>2650</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <f aca="false">D8/B8</f>
+        <v>0.3</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <f aca="false">D6+D7</f>
+        <v>795</v>
+      </c>
+      <c r="E8" s="12" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="10" t="n">
-        <v>795</v>
-      </c>
-      <c r="C9" s="10" t="n">
-        <v>14566.2351053328</v>
-      </c>
-      <c r="D9" s="11" t="n">
-        <f aca="false">B9/C9</f>
-        <v>0.0545782760096289</v>
-      </c>
-      <c r="E9" s="12" t="s">
+    </row>
+    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="B11" s="6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="C11" s="6" t="s">
         <v>17</v>
       </c>
+      <c r="D11" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="7" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C12" s="7" t="n">
+        <f aca="false">B6</f>
+        <v>1800</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <f aca="false">B12-C12</f>
+        <v>-200</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="A13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="B13" s="7" t="n">
+        <v>850</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <f aca="false">B7</f>
+        <v>850</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <f aca="false">B13-C13</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F13" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="H13" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="L13" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="M13" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="N13" s="6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>-19.58417776</v>
-      </c>
-      <c r="C14" s="7" t="n">
-        <v>-12.2</v>
-      </c>
-      <c r="D14" s="7" t="n">
-        <v>-0.525</v>
-      </c>
-      <c r="E14" s="7" t="n">
-        <v>-4.55378175</v>
-      </c>
-      <c r="F14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="7" t="n">
-        <f aca="false">SUM(B14:M14)</f>
-        <v>-36.86295951</v>
-      </c>
+      <c r="B14" s="10" t="n">
+        <f aca="false">B12+B13</f>
+        <v>2450</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <f aca="false">C12+C13</f>
+        <v>2650</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <f aca="false">B14-C14</f>
+        <v>-200</v>
+      </c>
+      <c r="E14" s="12"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <f aca="false">C8</f>
+        <v>0.3</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <f aca="false">B15-C15</f>
+        <v>0.02</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="10" t="n">
+        <f aca="false">B14*B15</f>
+        <v>784</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <f aca="false">D8</f>
+        <v>795</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <f aca="false">B16-C16</f>
+        <v>-11</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="B17" s="14" t="n">
+        <f aca="false">795/B14</f>
+        <v>0.324489795918367</v>
+      </c>
+      <c r="C17" s="15"/>
+      <c r="D17" s="15"/>
+      <c r="E17" s="15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0.88083585</v>
-      </c>
-      <c r="D15" s="7" t="n">
-        <v>37.16684613</v>
-      </c>
-      <c r="E15" s="7" t="n">
-        <v>4.45802033</v>
-      </c>
-      <c r="F15" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="7" t="n">
-        <v>43.63757336</v>
-      </c>
-      <c r="H15" s="7" t="n">
-        <v>7.51786912</v>
-      </c>
-      <c r="I15" s="7" t="n">
-        <v>0.939976</v>
-      </c>
-      <c r="N15" s="7" t="n">
-        <f aca="false">SUM(B15:M15)</f>
-        <v>94.60112079</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+      <c r="B22" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C22" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="D22" s="7" t="n">
+        <v>1246.86</v>
+      </c>
+      <c r="E22" s="7" t="n">
+        <v>1000</v>
+      </c>
+      <c r="F22" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="7" t="n">
-        <v>2.20404132</v>
-      </c>
-      <c r="D16" s="7" t="n">
-        <v>0.80646765</v>
-      </c>
-      <c r="E16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="7" t="n">
-        <v>1.74350512</v>
-      </c>
-      <c r="H16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="7" t="n">
-        <f aca="false">SUM(B16:M16)</f>
-        <v>4.75401409</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>351.73</v>
+      </c>
+      <c r="C23" s="10" t="n">
+        <v>354.4</v>
+      </c>
+      <c r="D23" s="10" t="n">
+        <v>332.41</v>
+      </c>
+      <c r="E23" s="10" t="n">
+        <f aca="false">E22*E24</f>
+        <v>360</v>
+      </c>
+      <c r="F23" s="12" t="s">
         <v>35</v>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="C17" s="7" t="n">
-        <v>21.5737716</v>
-      </c>
-      <c r="D17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="7" t="n">
-        <v>38.17544837</v>
-      </c>
-      <c r="H17" s="7" t="n">
-        <v>14.7602298</v>
-      </c>
-      <c r="I17" s="7" t="n">
-        <v>1.17900459</v>
-      </c>
-      <c r="N17" s="7" t="n">
-        <f aca="false">SUM(B17:M17)</f>
-        <v>75.68845436</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="J18" s="7" t="n">
-        <v>43.8894850443278</v>
-      </c>
-      <c r="K18" s="7" t="n">
-        <v>47.0923180264855</v>
-      </c>
-      <c r="L18" s="7" t="n">
-        <v>48.060136571781</v>
-      </c>
-      <c r="M18" s="7" t="n">
-        <v>55.1887770224611</v>
-      </c>
-      <c r="N18" s="7" t="n">
-        <f aca="false">SUM(B18:M18)</f>
-        <v>194.230716665055</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B19" s="10" t="n">
-        <f aca="false">SUM(B14:B18)</f>
-        <v>-19.58417776</v>
-      </c>
-      <c r="C19" s="10" t="n">
-        <f aca="false">SUM(C14:C18)</f>
-        <v>12.45864877</v>
-      </c>
-      <c r="D19" s="10" t="n">
-        <f aca="false">SUM(D14:D18)</f>
-        <v>37.44831378</v>
-      </c>
-      <c r="E19" s="10" t="n">
-        <f aca="false">SUM(E14:E18)</f>
-        <v>-0.0957614199999997</v>
-      </c>
-      <c r="F19" s="10" t="n">
-        <f aca="false">SUM(F14:F18)</f>
-        <v>0</v>
-      </c>
-      <c r="G19" s="10" t="n">
-        <f aca="false">SUM(G14:G18)</f>
-        <v>83.55652685</v>
-      </c>
-      <c r="H19" s="10" t="n">
-        <f aca="false">SUM(H14:H18)</f>
-        <v>22.27809892</v>
-      </c>
-      <c r="I19" s="10" t="n">
-        <f aca="false">SUM(I14:I18)</f>
-        <v>2.11898059</v>
-      </c>
-      <c r="J19" s="10" t="n">
-        <f aca="false">SUM(J14:J18)</f>
-        <v>43.8894850443278</v>
-      </c>
-      <c r="K19" s="10" t="n">
-        <f aca="false">SUM(K14:K18)</f>
-        <v>47.0923180264855</v>
-      </c>
-      <c r="L19" s="10" t="n">
-        <f aca="false">SUM(L14:L18)</f>
-        <v>48.060136571781</v>
-      </c>
-      <c r="M19" s="10" t="n">
-        <f aca="false">SUM(M14:M18)</f>
-        <v>55.1887770224611</v>
-      </c>
-      <c r="N19" s="10" t="n">
-        <f aca="false">SUM(N14:N18)</f>
-        <v>332.411346395055</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3"/>
-    </row>
-    <row r="22" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B24" s="8" t="n">
+        <f aca="false">B23/B22</f>
+        <v>0.35173</v>
+      </c>
+      <c r="C24" s="8" t="n">
+        <f aca="false">C23/C22</f>
+        <v>0.3544</v>
+      </c>
+      <c r="D24" s="8" t="n">
+        <f aca="false">D23/D22</f>
+        <v>0.266597693405836</v>
+      </c>
+      <c r="E24" s="8" t="n">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B29" s="8" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D29" s="16" t="n">
+        <f aca="false">(C29-B29)*100</f>
+        <v>-4</v>
+      </c>
+      <c r="E29" s="9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B24" s="7" t="n">
-        <v>711.782499521939</v>
-      </c>
-      <c r="C24" s="7" t="n">
-        <v>75.68845436</v>
-      </c>
-      <c r="D24" s="8" t="n">
-        <f aca="false">IFERROR(C24/B24,"")</f>
-        <v>0.10633649241283</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+      <c r="B30" s="8" t="n">
+        <f aca="false">B24</f>
+        <v>0.35173</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <f aca="false">C8</f>
+        <v>0.3</v>
+      </c>
+      <c r="D30" s="16" t="n">
+        <f aca="false">(C30-B30)*100</f>
+        <v>-5.17300000000001</v>
+      </c>
+      <c r="E30" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B25" s="7" t="n">
-        <v>190.761574310513</v>
-      </c>
-      <c r="C25" s="7" t="n">
-        <v>4.75401409</v>
-      </c>
-      <c r="D25" s="8" t="n">
-        <f aca="false">IFERROR(C25/B25,"")</f>
-        <v>0.0249212353545669</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B26" s="7" t="n">
-        <v>1484.31679755366</v>
-      </c>
-      <c r="C26" s="7" t="n">
+      <c r="B31" s="8" t="n">
+        <f aca="false">B24</f>
+        <v>0.35173</v>
+      </c>
+      <c r="C31" s="8" t="n">
+        <f aca="false">B17</f>
+        <v>0.324489795918367</v>
+      </c>
+      <c r="D31" s="16" t="n">
+        <f aca="false">(C31-B31)*100</f>
+        <v>-2.72402040816327</v>
+      </c>
+      <c r="E31" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G35" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="H35" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="K35" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L35" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="M35" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="N35" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>-19.58417776</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>-12.2</v>
+      </c>
+      <c r="D36" s="7" t="n">
+        <v>-0.525</v>
+      </c>
+      <c r="E36" s="7" t="n">
+        <v>-4.55378175</v>
+      </c>
+      <c r="F36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" s="7" t="n">
+        <f aca="false">SUM(B36:M36)</f>
+        <v>-36.86295951</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>0.88083585</v>
+      </c>
+      <c r="D37" s="7" t="n">
+        <v>37.16684613</v>
+      </c>
+      <c r="E37" s="7" t="n">
+        <v>4.45802033</v>
+      </c>
+      <c r="F37" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>43.63757336</v>
+      </c>
+      <c r="H37" s="7" t="n">
+        <v>7.51786912</v>
+      </c>
+      <c r="I37" s="7" t="n">
+        <v>0.939976</v>
+      </c>
+      <c r="N37" s="7" t="n">
+        <f aca="false">SUM(B37:M37)</f>
         <v>94.60112079</v>
-      </c>
-      <c r="D26" s="8" t="n">
-        <f aca="false">IFERROR(C26/B26,"")</f>
-        <v>0.0637337803802494</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C27" s="7" t="n">
-        <v>-36.86295951</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="B28" s="10" t="n">
-        <f aca="false">SUM(B24:B27)</f>
-        <v>2386.86087138611</v>
-      </c>
-      <c r="C28" s="10" t="n">
-        <f aca="false">SUM(C24:C27)</f>
-        <v>138.18062973</v>
-      </c>
-      <c r="D28" s="11" t="n">
-        <f aca="false">IFERROR(C28/B28,"")</f>
-        <v>0.0578922011695449</v>
-      </c>
-      <c r="E28" s="12" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="G32" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="I32" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="J32" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="K32" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="L32" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="M32" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="N32" s="6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="C33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="D33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="E33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="F33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="G33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="H33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="I33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="J33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="K33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="L33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="M33" s="10" t="n">
-        <v>66.25</v>
-      </c>
-      <c r="N33" s="10" t="n">
-        <f aca="false">SUM(B33:M33)</f>
-        <v>795</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3"/>
-    </row>
-    <row r="36" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B38" s="7" t="n">
-        <v>14566.2351053328</v>
-      </c>
-      <c r="C38" s="9" t="s">
-        <v>60</v>
+        <v>0</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>2.20404132</v>
+      </c>
+      <c r="D38" s="7" t="n">
+        <v>0.80646765</v>
+      </c>
+      <c r="E38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>1.74350512</v>
+      </c>
+      <c r="H38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="7" t="n">
+        <f aca="false">SUM(B38:M38)</f>
+        <v>4.75401409</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B39" s="8" t="n">
-        <v>0.430091554994713</v>
-      </c>
-      <c r="C39" s="9" t="s">
-        <v>62</v>
+        <v>67</v>
+      </c>
+      <c r="B39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C39" s="7" t="n">
+        <v>21.5737716</v>
+      </c>
+      <c r="D39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>38.17544837</v>
+      </c>
+      <c r="H39" s="7" t="n">
+        <v>14.7602298</v>
+      </c>
+      <c r="I39" s="7" t="n">
+        <v>1.17900459</v>
+      </c>
+      <c r="N39" s="7" t="n">
+        <f aca="false">SUM(B39:M39)</f>
+        <v>75.68845436</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B40" s="7" t="n">
-        <f aca="false">B38*B39</f>
-        <v>6264.81470687115</v>
+        <v>68</v>
+      </c>
+      <c r="J40" s="7" t="n">
+        <v>43.8894850443278</v>
+      </c>
+      <c r="K40" s="7" t="n">
+        <v>47.0923180264855</v>
+      </c>
+      <c r="L40" s="7" t="n">
+        <v>48.060136571781</v>
+      </c>
+      <c r="M40" s="7" t="n">
+        <v>55.1887770224611</v>
+      </c>
+      <c r="N40" s="7" t="n">
+        <f aca="false">SUM(B40:M40)</f>
+        <v>194.230716665055</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="B41" s="14" t="n">
-        <f aca="false">795/B40</f>
-        <v>0.126899204078304</v>
-      </c>
-      <c r="C41" s="15" t="s">
-        <v>65</v>
+      <c r="A41" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="B41" s="10" t="n">
+        <f aca="false">SUM(B36:B40)</f>
+        <v>-19.58417776</v>
+      </c>
+      <c r="C41" s="10" t="n">
+        <f aca="false">SUM(C36:C40)</f>
+        <v>12.45864877</v>
+      </c>
+      <c r="D41" s="10" t="n">
+        <f aca="false">SUM(D36:D40)</f>
+        <v>37.44831378</v>
+      </c>
+      <c r="E41" s="10" t="n">
+        <f aca="false">SUM(E36:E40)</f>
+        <v>-0.0957614199999997</v>
+      </c>
+      <c r="F41" s="10" t="n">
+        <f aca="false">SUM(F36:F40)</f>
+        <v>0</v>
+      </c>
+      <c r="G41" s="10" t="n">
+        <f aca="false">SUM(G36:G40)</f>
+        <v>83.55652685</v>
+      </c>
+      <c r="H41" s="10" t="n">
+        <f aca="false">SUM(H36:H40)</f>
+        <v>22.27809892</v>
+      </c>
+      <c r="I41" s="10" t="n">
+        <f aca="false">SUM(I36:I40)</f>
+        <v>2.11898059</v>
+      </c>
+      <c r="J41" s="10" t="n">
+        <f aca="false">SUM(J36:J40)</f>
+        <v>43.8894850443278</v>
+      </c>
+      <c r="K41" s="10" t="n">
+        <f aca="false">SUM(K36:K40)</f>
+        <v>47.0923180264855</v>
+      </c>
+      <c r="L41" s="10" t="n">
+        <f aca="false">SUM(L36:L40)</f>
+        <v>48.060136571781</v>
+      </c>
+      <c r="M41" s="10" t="n">
+        <f aca="false">SUM(M36:M40)</f>
+        <v>55.1887770224611</v>
+      </c>
+      <c r="N41" s="10" t="n">
+        <f aca="false">SUM(N36:N40)</f>
+        <v>332.411346395055</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="B42" s="16" t="n">
-        <f aca="false">B40*0.0578922011695449</f>
-        <v>362.683913300109</v>
-      </c>
-      <c r="C42" s="15" t="s">
-        <v>67</v>
+      <c r="A42" s="3"/>
+    </row>
+    <row r="43" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="C43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="D43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="E43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="F43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="G43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="H43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="I43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="J43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="K43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="L43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="M43" s="10" t="n">
+        <v>66.25</v>
+      </c>
+      <c r="N43" s="10" t="n">
+        <f aca="false">SUM(B43:M43)</f>
+        <v>795</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>
@@ -1747,12 +1821,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1760,32 +1834,32 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>392.559665831245</v>
@@ -1808,7 +1882,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>787.912447786132</v>
@@ -1831,7 +1905,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>419.527886382623</v>
@@ -1854,7 +1928,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">SUM(B6:B8)</f>
@@ -1875,7 +1949,7 @@
     </row>
     <row r="10" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1883,45 +1957,45 @@
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B14" s="7" t="n">
         <v>595.55</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B15" s="7" t="n">
         <v>404.45</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>1000</v>
@@ -1933,24 +2007,24 @@
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>7</v>
@@ -1958,7 +2032,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B20" s="7" t="n">
         <v>986.999999999999</v>
@@ -1975,12 +2049,12 @@
         <v>0.48273556231003</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B21" s="7" t="n">
         <v>530.702863852945</v>
@@ -1997,12 +2071,12 @@
         <v>0.426260090157773</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B22" s="7" t="n">
         <v>530.702863852945</v>
@@ -2019,12 +2093,12 @@
         <v>0.198825854880224</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>369.316632851684</v>
@@ -2043,7 +2117,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>900.019496704628</v>
@@ -2060,12 +2134,12 @@
         <v>0.495857354200569</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B25" s="7" t="n">
         <v>900.019496704628</v>
@@ -2084,7 +2158,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B26" s="7" t="n">
         <v>546.94153</v>
@@ -2101,12 +2175,12 @@
         <v>0.658677998626936</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2114,56 +2188,56 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>20</v>
+        <v>52</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>24</v>
+        <v>56</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>26</v>
+        <v>58</v>
       </c>
       <c r="J30" s="6" t="s">
-        <v>27</v>
+        <v>59</v>
       </c>
       <c r="K30" s="6" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>31</v>
+        <v>63</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B31" s="7" t="n">
         <v>16.9387687250432</v>
@@ -2208,7 +2282,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B32" s="7" t="n">
         <v>28.52889409</v>
@@ -2253,7 +2327,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B33" s="10" t="n">
         <f aca="false">B31-B32</f>
@@ -2310,7 +2384,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B34" s="8" t="n">
         <f aca="false">IFERROR(B33/B31,"")</f>
@@ -2367,7 +2441,7 @@
     </row>
     <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2375,15 +2449,15 @@
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>7</v>
@@ -2391,7 +2465,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B39" s="7" t="n">
         <v>282.49799362</v>
@@ -2399,7 +2473,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B40" s="7" t="n">
         <v>109.84879112</v>
@@ -2407,7 +2481,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B41" s="7" t="n">
         <v>31.31843725</v>
@@ -2415,7 +2489,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B42" s="7" t="n">
         <v>19.726605</v>
@@ -2423,7 +2497,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B43" s="7" t="n">
         <v>16.0624436</v>
@@ -2431,7 +2505,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B44" s="7" t="n">
         <v>9.92231206</v>
@@ -2439,7 +2513,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B45" s="7" t="n">
         <v>2.15214708</v>
@@ -2447,7 +2521,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B46" s="7" t="n">
         <v>-46.34583669</v>
@@ -2455,7 +2529,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B47" s="7" t="n">
         <v>-120.6984392</v>
@@ -2463,7 +2537,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>50</v>
+        <v>129</v>
       </c>
       <c r="B48" s="10" t="n">
         <f aca="false">SUM(B39:B47)</f>
@@ -2476,35 +2550,35 @@
     </row>
     <row r="50" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="B52" s="7" t="n">
         <v>267.84</v>
@@ -2529,7 +2603,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B53" s="7" t="n">
         <v>149.76153</v>
@@ -2554,7 +2628,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B54" s="7" t="n">
         <v>88</v>
@@ -2579,7 +2653,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="B55" s="7" t="n">
         <v>41.34</v>
@@ -2604,7 +2678,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B56" s="10" t="n">
         <f aca="false">SUM(B52:B55)</f>
@@ -2636,30 +2710,30 @@
     </row>
     <row r="58" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="F58" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G58" s="6" t="s">
         <v>135</v>
-      </c>
-      <c r="B58" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D58" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="E58" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="F58" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="G58" s="6" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="B59" s="7" t="n">
         <v>130.8826</v>
@@ -2684,7 +2758,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B60" s="7" t="n">
         <v>117.71</v>
@@ -2709,7 +2783,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B61" s="7" t="n">
         <v>88</v>
@@ -2734,7 +2808,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="B62" s="7" t="n">
         <v>72.5556</v>
@@ -2759,7 +2833,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="B63" s="7" t="n">
         <v>50</v>
@@ -2784,7 +2858,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B64" s="7" t="n">
         <v>41.34</v>
@@ -2809,7 +2883,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B65" s="7" t="n">
         <v>23.50433</v>
@@ -2834,7 +2908,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="B66" s="7" t="n">
         <v>12.359</v>
@@ -2859,7 +2933,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B67" s="7" t="n">
         <v>6</v>
@@ -2884,7 +2958,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="B68" s="7" t="n">
         <v>4.59</v>
@@ -2909,7 +2983,7 @@
     </row>
     <row r="69" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2917,32 +2991,32 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="B73" s="7" t="n">
         <v>768.821180909195</v>
@@ -2965,7 +3039,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="B74" s="7" t="n">
         <v>192.791639187493</v>
@@ -2988,7 +3062,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="B75" s="7" t="n">
         <v>18.942306944518</v>
@@ -3011,7 +3085,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B76" s="7" t="n">
         <v>6.44487295879252</v>
@@ -3034,7 +3108,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="B77" s="10" t="n">
         <f aca="false">SUM(B73:B76)</f>
@@ -3053,12 +3127,12 @@
     </row>
     <row r="78" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3066,23 +3140,23 @@
     </row>
     <row r="81" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="5" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B83" s="7" t="n">
         <v>531.102863852944</v>
@@ -3094,7 +3168,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>164</v>
+        <v>8</v>
       </c>
       <c r="B84" s="7" t="n">
         <v>-0.4</v>
@@ -3106,7 +3180,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B85" s="10" t="n">
         <f aca="false">SUM(B83:B84)</f>
@@ -3119,21 +3193,21 @@
     </row>
     <row r="87" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B88" s="7" t="n">
         <v>221.156488366715</v>
@@ -3148,7 +3222,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B89" s="7" t="n">
         <v>84.3864815491803</v>
@@ -3163,7 +3237,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B90" s="7" t="n">
         <v>74.038</v>
@@ -3178,7 +3252,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B91" s="7" t="n">
         <v>50.85</v>
@@ -3193,7 +3267,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B92" s="7" t="n">
         <v>40.85</v>
@@ -3208,7 +3282,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B93" s="7" t="n">
         <v>26.3338573770492</v>
@@ -3223,7 +3297,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="B94" s="7" t="n">
         <v>9.57</v>
@@ -3238,7 +3312,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B95" s="7" t="n">
         <v>5.50803083</v>
@@ -3253,7 +3327,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="B96" s="7" t="n">
         <v>5.2</v>
@@ -3268,7 +3342,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B97" s="7" t="n">
         <v>5.06</v>
@@ -3283,7 +3357,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="B98" s="7" t="n">
         <v>4</v>
@@ -3298,7 +3372,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B99" s="7" t="n">
         <v>2.05</v>
@@ -3313,7 +3387,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="B100" s="7" t="n">
         <v>1.19000573</v>
@@ -3328,7 +3402,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="B101" s="7" t="n">
         <v>0.51</v>
@@ -3343,7 +3417,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B102" s="10" t="n">
         <f aca="false">SUM(B88:B101)</f>
@@ -3357,12 +3431,12 @@
     </row>
     <row r="103" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3370,26 +3444,26 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="5" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="B108" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C108" s="7" t="n">
         <v>61.0599999999998</v>
@@ -3397,10 +3471,10 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="B109" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C109" s="7" t="n">
         <v>53.0435999999999</v>
@@ -3408,10 +3482,10 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C110" s="7" t="n">
         <v>50</v>
@@ -3419,10 +3493,10 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="3" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C111" s="7" t="n">
         <v>33.9</v>
@@ -3430,10 +3504,10 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B112" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C112" s="7" t="n">
         <v>33.236361</v>
@@ -3441,10 +3515,10 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C113" s="7" t="n">
         <v>25.3501545</v>
@@ -3452,10 +3526,10 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="B114" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C114" s="7" t="n">
         <v>21.6000445</v>
@@ -3463,10 +3537,10 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="3" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
       <c r="B115" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C115" s="7" t="n">
         <v>20.15022926</v>
@@ -3474,10 +3548,10 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="B116" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C116" s="7" t="n">
         <v>18</v>
@@ -3485,10 +3559,10 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="3" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="B117" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C117" s="7" t="n">
         <v>14.15895</v>

</xml_diff>

<commit_message>
Approvers' backup: DMP sheet aligned with business answer (directions 2026 vs 2027, margin bridge, model reconciliation)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TjyVtBMeKRjjZMJmWM6RZp
</commit_message>
<xml_diff>
--- a/BU2027_вопросы_согласующих_база.xlsx
+++ b/BU2027_вопросы_согласующих_база.xlsx
@@ -9,7 +9,8 @@
   </bookViews>
   <sheets>
     <sheet name="1. Вознаграждения РА" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="2. DMP + Online" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="2. DMP — ответ бизнеса" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Справка DMP (внутр.)" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="267">
   <si>
     <t xml:space="preserve">1. Вознаграждения рекламным агентствам (суперкомиссия, СК): 2026 vs 2027, млн руб. без НДС</t>
   </si>
@@ -239,6 +240,219 @@
     <t xml:space="preserve">2026: янв–авг — факт начислений (премии РА признаются по итогам периодов, помесячная динамика неравномерна); сен–дек — прогноз мастера августа. 2027 — 795 / 12.</t>
   </si>
   <si>
+    <t xml:space="preserve">2. DMP + Online: разбивка по направлениям 2026 vs 2027 (данные бизнеса), млн руб. без НДС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Источник: ответ бизнеса (команда DMP). Итоги сверены с бюджетной моделью cons 16.10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 Выручка, маржинальность и затраты на трафик по направлениям</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Направление</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржа 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Трафик 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржа 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Трафик 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ выручки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Δ маржи, п.п.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Комментарий бизнеса</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пакеты и Онлайн+ТВ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржинальность без изменений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Баннеры и OLV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рост маржинальности за счёт улучшения условий закупки (рост объёмов)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Новые площадки (SmartTV, Авито, МР)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Снижение маржинальности за счёт ухода ТГ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Онлайн на широких сегментах (новое)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Новые пакеты 2027 по запросу маркетинга и крупных поставщиков (Pepsi, P&amp;G, Mondelez)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого по направлениям</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого по модели (P&amp;L)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржинальность 48% → 37,5%: −10,7 п.п.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Расхождение: направления − модель</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка по направлениям не сходится с итогом: 2026 — на 24 млн меньше, 2027 — на 11 млн больше</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Формулировка «маржинальность снижается на 11%» — это 11 п.п. (48% → 37,5%), а не 11%. Предлагаем писать «на ~11 п.п.».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 Мост маржинальности 2026 → 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Шаг</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржинальность</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржинальность 2026 (модель)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">987 / 511</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027 без «онлайна на широких сегментах»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Действующие направления: баннеры +1 п.п., новые площадки −6,5 п.п. (уход ТГ), изменение структуры</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027 с «онлайном на широких сегментах»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Новые пакеты 440 млн с маржой 17,5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итог 2027 по модели (с учётом расхождения разбивки)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сумма направлений бизнеса больше итога модели на 11 млн</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого изменение</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~70% снижения маржинальности (−7,7 из −10,8 п.п.) дают новые пакеты на широких сегментах; действующие направления дают −2,6 п.п., в основном новые площадки (уход ТГ).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3 Прирост выручки и денег, остающихся Магниту (к вопросу «20 копеек с рубля»)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Блок</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прирост выручки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прирост маржи (выручка − трафик)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржа на 1 руб. прироста</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Действующие направления</t>
+  </si>
+  <si>
+    <t xml:space="preserve">По направлениям бизнеса (без расхождения с итогом модели)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Онлайн на широких сегментах</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого DMP+Online (модель)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">613 → +124: так считают согласующие</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4 Сверка с бюджетной моделью: в модели другая разбивка по направлениям</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Направление в модели (лист DMP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В модели «широкие сегменты» не выделены: часть, видимо, внутри пакетов (маржа 25%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого модель</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итоги модели и бизнеса совпадают (1 600 / 1 000 / 37,5%), разбивка — нет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Закупка трафика в реестре: DMP+Online (ЦМ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отдельная строка реестра (ответственный — Ардаширов Д.). Похоже на «широкие сегменты по запросу маркетинга» (расход 363) — нужно подтвердить</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.5 К тезису «все источники — поставщики, не РА; СК не выплачивается»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Показатель, факт 8М 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Значение</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка DMP+Online, всего</t>
+  </si>
+  <si>
+    <t xml:space="preserve">«Расшифровка» мастера</t>
+  </si>
+  <si>
+    <t xml:space="preserve">в т.ч. от поставщиков</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100% — подтверждает тезис бизнеса</t>
+  </si>
+  <si>
+    <t xml:space="preserve">в т.ч. проведено через РА (реальное направление «(РА)»)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~29% выручки DMP+Online 8М шло через агентства</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Премии РА: data/online, начислено</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Небольшие премии РА по DMP в 2026 начислялись</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027: DMP в базе СК</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В расчёте СК 2027 база — не поставщики и бренд-бюджеты; DMP не входит</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Для 2026 тезис «не через РА, СК не выплачивается» фактом не подтверждается полностью. Безопаснее формулировка: «в бюджете 2027 СК по DMP не закладывается; бюджеты — поставщиков».</t>
+  </si>
+  <si>
     <t xml:space="preserve">2. DMP + Online: выручка, закупка трафика и маржинальность, млн руб. без НДС</t>
   </si>
   <si>
@@ -248,15 +462,9 @@
     <t xml:space="preserve">2.1 BU 2027 по направлениям (план команды DMP)</t>
   </si>
   <si>
-    <t xml:space="preserve">Направление</t>
-  </si>
-  <si>
     <t xml:space="preserve">Выручка</t>
   </si>
   <si>
-    <t xml:space="preserve">Маржинальность</t>
-  </si>
-  <si>
     <t xml:space="preserve">Закупка трафика</t>
   </si>
   <si>
@@ -264,12 +472,6 @@
   </si>
   <si>
     <t xml:space="preserve">Доля выручки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Пакеты и Онлайн+ТВ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Баннеры и OLV</t>
   </si>
   <si>
     <t xml:space="preserve">Развитие новых площадок (SmartTV, Авито, МР)</t>
@@ -627,12 +829,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0;[RED]\-#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
     <numFmt numFmtId="167" formatCode="0.0"/>
-    <numFmt numFmtId="168" formatCode="0"/>
+    <numFmt numFmtId="168" formatCode="#,##0;[RED]\-#,##0"/>
+    <numFmt numFmtId="169" formatCode="0.00"/>
+    <numFmt numFmtId="170" formatCode="0"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -734,7 +938,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -808,6 +1012,30 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1811,6 +2039,730 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:J45"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="44"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="J1" s="3"/>
+    </row>
+    <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="J3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="J4" s="3"/>
+    </row>
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="17" t="n">
+        <v>220</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <f aca="false">IF(B6="","",B6*(1-C6))</f>
+        <v>132</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>292</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G6" s="17" t="n">
+        <f aca="false">E6*(1-F6)</f>
+        <v>175.2</v>
+      </c>
+      <c r="H6" s="17" t="n">
+        <f aca="false">E6-N(B6)</f>
+        <v>72</v>
+      </c>
+      <c r="I6" s="7" t="n">
+        <f aca="false">IF(C6="","",(F6-C6)*100)</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="17" t="n">
+        <v>505</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D7" s="17" t="n">
+        <f aca="false">IF(B7="","",B7*(1-C7))</f>
+        <v>262.6</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>589</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="G7" s="17" t="n">
+        <f aca="false">E7*(1-F7)</f>
+        <v>300.39</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <f aca="false">E7-N(B7)</f>
+        <v>84</v>
+      </c>
+      <c r="I7" s="7" t="n">
+        <f aca="false">IF(C7="","",(F7-C7)*100)</f>
+        <v>1</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B8" s="17" t="n">
+        <v>238</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="D8" s="17" t="n">
+        <f aca="false">IF(B8="","",B8*(1-C8))</f>
+        <v>116.62</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>290</v>
+      </c>
+      <c r="F8" s="8" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="G8" s="17" t="n">
+        <f aca="false">E8*(1-F8)</f>
+        <v>160.95</v>
+      </c>
+      <c r="H8" s="17" t="n">
+        <f aca="false">E8-N(B8)</f>
+        <v>52</v>
+      </c>
+      <c r="I8" s="7" t="n">
+        <f aca="false">IF(C8="","",(F8-C8)*100)</f>
+        <v>-6.5</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B9" s="17"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="17" t="str">
+        <f aca="false">IF(B9="","",B9*(1-C9))</f>
+        <v/>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>440</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="G9" s="17" t="n">
+        <f aca="false">E9*(1-F9)</f>
+        <v>363</v>
+      </c>
+      <c r="H9" s="17" t="n">
+        <f aca="false">E9-N(B9)</f>
+        <v>440</v>
+      </c>
+      <c r="I9" s="7" t="str">
+        <f aca="false">IF(C9="","",(F9-C9)*100)</f>
+        <v/>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="B10" s="18" t="n">
+        <f aca="false">SUM(B6:B9)</f>
+        <v>963</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <f aca="false">1-D10/B10</f>
+        <v>0.469138110072689</v>
+      </c>
+      <c r="D10" s="18" t="n">
+        <f aca="false">SUM(D6:D9)</f>
+        <v>511.22</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <f aca="false">SUM(E6:E9)</f>
+        <v>1611</v>
+      </c>
+      <c r="F10" s="11" t="n">
+        <f aca="false">1-G10/E10</f>
+        <v>0.379553072625698</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <f aca="false">SUM(G6:G9)</f>
+        <v>999.54</v>
+      </c>
+      <c r="H10" s="18" t="n">
+        <f aca="false">E10-B10</f>
+        <v>648</v>
+      </c>
+      <c r="I10" s="10" t="n">
+        <f aca="false">(F10-C10)*100</f>
+        <v>-8.95850374469911</v>
+      </c>
+      <c r="J10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B11" s="18" t="n">
+        <v>987</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <f aca="false">1-D11/B11</f>
+        <v>0.48273556231003</v>
+      </c>
+      <c r="D11" s="18" t="n">
+        <v>510.54</v>
+      </c>
+      <c r="E11" s="18" t="n">
+        <v>1600</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <f aca="false">1-G11/E11</f>
+        <v>0.375</v>
+      </c>
+      <c r="G11" s="18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="H11" s="18" t="n">
+        <f aca="false">E11-B11</f>
+        <v>613</v>
+      </c>
+      <c r="I11" s="10" t="n">
+        <f aca="false">(F11-C11)*100</f>
+        <v>-10.773556231003</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="B12" s="19" t="n">
+        <f aca="false">B10-B11</f>
+        <v>-24</v>
+      </c>
+      <c r="C12" s="15"/>
+      <c r="D12" s="20" t="n">
+        <f aca="false">D10-D11</f>
+        <v>0.680000000000007</v>
+      </c>
+      <c r="E12" s="19" t="n">
+        <f aca="false">E10-E11</f>
+        <v>11</v>
+      </c>
+      <c r="F12" s="15"/>
+      <c r="G12" s="20" t="n">
+        <f aca="false">G10-G11</f>
+        <v>-0.460000000000036</v>
+      </c>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3"/>
+      <c r="J14" s="3"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="J15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="8" t="n">
+        <f aca="false">C11</f>
+        <v>0.48273556231003</v>
+      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="J17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="8" t="n">
+        <f aca="false">1-SUM(G6:G8)/SUM(E6:E8)</f>
+        <v>0.456413321947054</v>
+      </c>
+      <c r="C18" s="7" t="n">
+        <f aca="false">(B18-B17)*100</f>
+        <v>-2.63222403629765</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="J18" s="3"/>
+    </row>
+    <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="B19" s="8" t="n">
+        <f aca="false">F10</f>
+        <v>0.379553072625698</v>
+      </c>
+      <c r="C19" s="7" t="n">
+        <f aca="false">(B19-B18)*100</f>
+        <v>-7.68602493213555</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="J19" s="3"/>
+    </row>
+    <row r="20" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="B20" s="8" t="n">
+        <f aca="false">F11</f>
+        <v>0.375</v>
+      </c>
+      <c r="C20" s="7" t="n">
+        <f aca="false">(B20-B19)*100</f>
+        <v>-0.455307262569837</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="J20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="B21" s="12"/>
+      <c r="C21" s="10" t="n">
+        <f aca="false">(B20-B17)*100</f>
+        <v>-10.773556231003</v>
+      </c>
+      <c r="D21" s="4"/>
+      <c r="J21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="J22" s="3"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3"/>
+      <c r="J23" s="3"/>
+    </row>
+    <row r="24" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="J24" s="3"/>
+    </row>
+    <row r="25" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J25" s="3"/>
+    </row>
+    <row r="26" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="B26" s="17" t="n">
+        <f aca="false">SUM(E6:E8)-SUM(B6:B8)</f>
+        <v>208</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <f aca="false">(SUM(E6:E8)-SUM(G6:G8))-(SUM(B6:B8)-SUM(D6:D8))</f>
+        <v>82.6800000000001</v>
+      </c>
+      <c r="D26" s="21" t="n">
+        <f aca="false">C26/B26</f>
+        <v>0.3975</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="J26" s="3"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" s="17" t="n">
+        <f aca="false">E9</f>
+        <v>440</v>
+      </c>
+      <c r="C27" s="17" t="n">
+        <f aca="false">E9-G9</f>
+        <v>77</v>
+      </c>
+      <c r="D27" s="21" t="n">
+        <f aca="false">C27/B27</f>
+        <v>0.175</v>
+      </c>
+      <c r="E27" s="3"/>
+      <c r="J27" s="3"/>
+    </row>
+    <row r="28" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="B28" s="18" t="n">
+        <f aca="false">E11-B11</f>
+        <v>613</v>
+      </c>
+      <c r="C28" s="18" t="n">
+        <f aca="false">(E11-G11)-(B11-D11)</f>
+        <v>123.54</v>
+      </c>
+      <c r="D28" s="22" t="n">
+        <f aca="false">C28/B28</f>
+        <v>0.201533442088091</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="J28" s="3"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3"/>
+      <c r="J29" s="3"/>
+    </row>
+    <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="J30" s="3"/>
+    </row>
+    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E31" s="5"/>
+      <c r="F31" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="J31" s="3"/>
+    </row>
+    <row r="32" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B32" s="17" t="n">
+        <v>392.56</v>
+      </c>
+      <c r="C32" s="8" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D32" s="17" t="n">
+        <v>294.54</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="J32" s="3"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B33" s="17" t="n">
+        <v>787.91</v>
+      </c>
+      <c r="C33" s="8" t="n">
+        <v>0.404</v>
+      </c>
+      <c r="D33" s="17" t="n">
+        <v>469.38</v>
+      </c>
+      <c r="F33" s="3"/>
+      <c r="J33" s="3"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B34" s="17" t="n">
+        <v>419.53</v>
+      </c>
+      <c r="C34" s="8" t="n">
+        <v>0.437</v>
+      </c>
+      <c r="D34" s="17" t="n">
+        <v>236.08</v>
+      </c>
+      <c r="F34" s="3"/>
+      <c r="J34" s="3"/>
+    </row>
+    <row r="35" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="B35" s="18" t="n">
+        <v>1600</v>
+      </c>
+      <c r="C35" s="11" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="D35" s="18" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E35" s="12"/>
+      <c r="F35" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="J35" s="3"/>
+    </row>
+    <row r="36" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="B36" s="19"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="19" t="n">
+        <v>404.45</v>
+      </c>
+      <c r="E36" s="15"/>
+      <c r="F36" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="J36" s="3"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3"/>
+      <c r="J37" s="3"/>
+    </row>
+    <row r="38" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="J38" s="3"/>
+    </row>
+    <row r="39" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J39" s="3"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B40" s="7" t="n">
+        <v>530.7</v>
+      </c>
+      <c r="C40" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="J40" s="3"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B41" s="7" t="n">
+        <v>531.1</v>
+      </c>
+      <c r="C41" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="J41" s="3"/>
+    </row>
+    <row r="42" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>136</v>
+      </c>
+      <c r="B42" s="20" t="n">
+        <v>153.5</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="J42" s="3"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="B43" s="20" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="J43" s="3"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B44" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C44" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="J44" s="3"/>
+    </row>
+    <row r="45" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="J45" s="3"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:N117"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -1821,12 +2773,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>73</v>
+        <v>144</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1834,7 +2786,7 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>74</v>
+        <v>145</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1842,24 +2794,24 @@
         <v>75</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>76</v>
+        <v>146</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>78</v>
+        <v>147</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>79</v>
+        <v>148</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>80</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>392.559665831245</v>
@@ -1882,7 +2834,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>787.912447786132</v>
@@ -1905,7 +2857,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>83</v>
+        <v>150</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>419.527886382623</v>
@@ -1928,7 +2880,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>84</v>
+        <v>151</v>
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">SUM(B6:B8)</f>
@@ -1949,7 +2901,7 @@
     </row>
     <row r="10" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>85</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1957,45 +2909,45 @@
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>86</v>
+        <v>153</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>87</v>
+        <v>154</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>88</v>
+        <v>155</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>89</v>
+        <v>156</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>90</v>
+        <v>157</v>
       </c>
       <c r="B14" s="7" t="n">
         <v>595.55</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>91</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>92</v>
+        <v>159</v>
       </c>
       <c r="B15" s="7" t="n">
         <v>404.45</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>93</v>
+        <v>160</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>94</v>
+        <v>161</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>1000</v>
@@ -2007,24 +2959,24 @@
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>95</v>
+        <v>162</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>96</v>
+        <v>163</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>76</v>
+        <v>146</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>97</v>
+        <v>164</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>79</v>
+        <v>148</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>7</v>
@@ -2032,7 +2984,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>98</v>
+        <v>165</v>
       </c>
       <c r="B20" s="7" t="n">
         <v>986.999999999999</v>
@@ -2049,12 +3001,12 @@
         <v>0.48273556231003</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>99</v>
+        <v>166</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>100</v>
+        <v>167</v>
       </c>
       <c r="B21" s="7" t="n">
         <v>530.702863852945</v>
@@ -2071,12 +3023,12 @@
         <v>0.426260090157773</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>101</v>
+        <v>168</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>102</v>
+        <v>169</v>
       </c>
       <c r="B22" s="7" t="n">
         <v>530.702863852945</v>
@@ -2093,12 +3045,12 @@
         <v>0.198825854880224</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>103</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>104</v>
+        <v>171</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>369.316632851684</v>
@@ -2117,7 +3069,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>105</v>
+        <v>172</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>900.019496704628</v>
@@ -2134,12 +3086,12 @@
         <v>0.495857354200569</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>106</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>107</v>
+        <v>174</v>
       </c>
       <c r="B25" s="7" t="n">
         <v>900.019496704628</v>
@@ -2158,7 +3110,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>108</v>
+        <v>175</v>
       </c>
       <c r="B26" s="7" t="n">
         <v>546.94153</v>
@@ -2175,12 +3127,12 @@
         <v>0.658677998626936</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>109</v>
+        <v>176</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>110</v>
+        <v>177</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2188,7 +3140,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>111</v>
+        <v>178</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2237,7 +3189,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>112</v>
+        <v>179</v>
       </c>
       <c r="B31" s="7" t="n">
         <v>16.9387687250432</v>
@@ -2282,7 +3234,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>113</v>
+        <v>180</v>
       </c>
       <c r="B32" s="7" t="n">
         <v>28.52889409</v>
@@ -2327,7 +3279,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>114</v>
+        <v>181</v>
       </c>
       <c r="B33" s="10" t="n">
         <f aca="false">B31-B32</f>
@@ -2384,7 +3336,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>115</v>
+        <v>182</v>
       </c>
       <c r="B34" s="8" t="n">
         <f aca="false">IFERROR(B33/B31,"")</f>
@@ -2441,7 +3393,7 @@
     </row>
     <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>116</v>
+        <v>183</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2449,15 +3401,15 @@
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>117</v>
+        <v>184</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>118</v>
+        <v>185</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>119</v>
+        <v>186</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>7</v>
@@ -2465,7 +3417,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>120</v>
+        <v>187</v>
       </c>
       <c r="B39" s="7" t="n">
         <v>282.49799362</v>
@@ -2473,7 +3425,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>121</v>
+        <v>188</v>
       </c>
       <c r="B40" s="7" t="n">
         <v>109.84879112</v>
@@ -2481,7 +3433,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>122</v>
+        <v>189</v>
       </c>
       <c r="B41" s="7" t="n">
         <v>31.31843725</v>
@@ -2489,7 +3441,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>123</v>
+        <v>190</v>
       </c>
       <c r="B42" s="7" t="n">
         <v>19.726605</v>
@@ -2497,7 +3449,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>124</v>
+        <v>191</v>
       </c>
       <c r="B43" s="7" t="n">
         <v>16.0624436</v>
@@ -2505,7 +3457,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>125</v>
+        <v>192</v>
       </c>
       <c r="B44" s="7" t="n">
         <v>9.92231206</v>
@@ -2513,7 +3465,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>126</v>
+        <v>193</v>
       </c>
       <c r="B45" s="7" t="n">
         <v>2.15214708</v>
@@ -2521,7 +3473,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>127</v>
+        <v>194</v>
       </c>
       <c r="B46" s="7" t="n">
         <v>-46.34583669</v>
@@ -2529,7 +3481,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>128</v>
+        <v>195</v>
       </c>
       <c r="B47" s="7" t="n">
         <v>-120.6984392</v>
@@ -2537,7 +3489,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>129</v>
+        <v>196</v>
       </c>
       <c r="B48" s="10" t="n">
         <f aca="false">SUM(B39:B47)</f>
@@ -2550,35 +3502,35 @@
     </row>
     <row r="50" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>130</v>
+        <v>197</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>131</v>
+        <v>198</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>76</v>
+        <v>146</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>132</v>
+        <v>199</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>133</v>
+        <v>200</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>134</v>
+        <v>201</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>135</v>
+        <v>202</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>136</v>
+        <v>203</v>
       </c>
       <c r="B52" s="7" t="n">
         <v>267.84</v>
@@ -2597,13 +3549,13 @@
         <f aca="false">IFERROR(1-E52/B52,"")</f>
         <v>0.639477572004224</v>
       </c>
-      <c r="G52" s="17" t="n">
+      <c r="G52" s="23" t="n">
         <v>75</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>137</v>
+        <v>204</v>
       </c>
       <c r="B53" s="7" t="n">
         <v>149.76153</v>
@@ -2622,13 +3574,13 @@
         <f aca="false">IFERROR(1-E53/B53,"")</f>
         <v>0.75765705792135</v>
       </c>
-      <c r="G53" s="17" t="n">
+      <c r="G53" s="23" t="n">
         <v>157</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>138</v>
+        <v>205</v>
       </c>
       <c r="B54" s="7" t="n">
         <v>88</v>
@@ -2647,13 +3599,13 @@
         <f aca="false">IFERROR(1-E54/B54,"")</f>
         <v>0.487682909899352</v>
       </c>
-      <c r="G54" s="17" t="n">
+      <c r="G54" s="23" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>139</v>
+        <v>206</v>
       </c>
       <c r="B55" s="7" t="n">
         <v>41.34</v>
@@ -2672,13 +3624,13 @@
         <f aca="false">IFERROR(1-E55/B55,"")</f>
         <v>0.788502737784228</v>
       </c>
-      <c r="G55" s="17" t="n">
+      <c r="G55" s="23" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>94</v>
+        <v>161</v>
       </c>
       <c r="B56" s="10" t="n">
         <f aca="false">SUM(B52:B55)</f>
@@ -2700,7 +3652,7 @@
         <f aca="false">IFERROR(1-E56/B56,"")</f>
         <v>0.658677998626936</v>
       </c>
-      <c r="G56" s="18" t="n">
+      <c r="G56" s="24" t="n">
         <f aca="false">SUM(G52:G55)</f>
         <v>280</v>
       </c>
@@ -2710,30 +3662,30 @@
     </row>
     <row r="58" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>140</v>
+        <v>207</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>76</v>
+        <v>146</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>132</v>
+        <v>199</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>133</v>
+        <v>200</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>134</v>
+        <v>201</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>135</v>
+        <v>202</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>141</v>
+        <v>208</v>
       </c>
       <c r="B59" s="7" t="n">
         <v>130.8826</v>
@@ -2752,13 +3704,13 @@
         <f aca="false">IFERROR(1-E59/B59,"")</f>
         <v>0.725782153089869</v>
       </c>
-      <c r="G59" s="17" t="n">
+      <c r="G59" s="23" t="n">
         <v>134</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>142</v>
+        <v>209</v>
       </c>
       <c r="B60" s="7" t="n">
         <v>117.71</v>
@@ -2777,13 +3729,13 @@
         <f aca="false">IFERROR(1-E60/B60,"")</f>
         <v>0.752562215067636</v>
       </c>
-      <c r="G60" s="17" t="n">
+      <c r="G60" s="23" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>143</v>
+        <v>210</v>
       </c>
       <c r="B61" s="7" t="n">
         <v>88</v>
@@ -2802,13 +3754,13 @@
         <f aca="false">IFERROR(1-E61/B61,"")</f>
         <v>0.487682909899352</v>
       </c>
-      <c r="G61" s="17" t="n">
+      <c r="G61" s="23" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>144</v>
+        <v>211</v>
       </c>
       <c r="B62" s="7" t="n">
         <v>72.5556</v>
@@ -2827,13 +3779,13 @@
         <f aca="false">IFERROR(1-E62/B62,"")</f>
         <v>0.612268256206275</v>
       </c>
-      <c r="G62" s="17" t="n">
+      <c r="G62" s="23" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>145</v>
+        <v>212</v>
       </c>
       <c r="B63" s="7" t="n">
         <v>50</v>
@@ -2852,13 +3804,13 @@
         <f aca="false">IFERROR(1-E63/B63,"")</f>
         <v>0.4466189338</v>
       </c>
-      <c r="G63" s="17" t="n">
+      <c r="G63" s="23" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>146</v>
+        <v>213</v>
       </c>
       <c r="B64" s="7" t="n">
         <v>41.34</v>
@@ -2877,13 +3829,13 @@
         <f aca="false">IFERROR(1-E64/B64,"")</f>
         <v>0.788502737784228</v>
       </c>
-      <c r="G64" s="17" t="n">
+      <c r="G64" s="23" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>147</v>
+        <v>214</v>
       </c>
       <c r="B65" s="7" t="n">
         <v>23.50433</v>
@@ -2902,13 +3854,13 @@
         <f aca="false">IFERROR(1-E65/B65,"")</f>
         <v>0.589605352698843</v>
       </c>
-      <c r="G65" s="17" t="n">
+      <c r="G65" s="23" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>148</v>
+        <v>215</v>
       </c>
       <c r="B66" s="7" t="n">
         <v>12.359</v>
@@ -2927,13 +3879,13 @@
         <f aca="false">IFERROR(1-E66/B66,"")</f>
         <v>0.999979091350433</v>
       </c>
-      <c r="G66" s="17" t="n">
+      <c r="G66" s="23" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>149</v>
+        <v>216</v>
       </c>
       <c r="B67" s="7" t="n">
         <v>6</v>
@@ -2952,13 +3904,13 @@
         <f aca="false">IFERROR(1-E67/B67,"")</f>
         <v>0.6013</v>
       </c>
-      <c r="G67" s="17" t="n">
+      <c r="G67" s="23" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>150</v>
+        <v>217</v>
       </c>
       <c r="B68" s="7" t="n">
         <v>4.59</v>
@@ -2977,13 +3929,13 @@
         <f aca="false">IFERROR(1-E68/B68,"")</f>
         <v>0.99998731590414</v>
       </c>
-      <c r="G68" s="17" t="n">
+      <c r="G68" s="23" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>151</v>
+        <v>218</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2991,32 +3943,32 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>152</v>
+        <v>219</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>153</v>
+        <v>220</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>154</v>
+        <v>221</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>155</v>
+        <v>222</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>156</v>
+        <v>223</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>155</v>
+        <v>222</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>157</v>
+        <v>224</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>158</v>
+        <v>225</v>
       </c>
       <c r="B73" s="7" t="n">
         <v>768.821180909195</v>
@@ -3039,7 +3991,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>159</v>
+        <v>226</v>
       </c>
       <c r="B74" s="7" t="n">
         <v>192.791639187493</v>
@@ -3062,7 +4014,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>160</v>
+        <v>227</v>
       </c>
       <c r="B75" s="7" t="n">
         <v>18.942306944518</v>
@@ -3085,7 +4037,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>161</v>
+        <v>228</v>
       </c>
       <c r="B76" s="7" t="n">
         <v>6.44487295879252</v>
@@ -3108,7 +4060,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>162</v>
+        <v>229</v>
       </c>
       <c r="B77" s="10" t="n">
         <f aca="false">SUM(B73:B76)</f>
@@ -3127,12 +4079,12 @@
     </row>
     <row r="78" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>163</v>
+        <v>230</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>164</v>
+        <v>231</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3140,23 +4092,23 @@
     </row>
     <row r="81" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="s">
-        <v>165</v>
+        <v>232</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="5" t="s">
-        <v>166</v>
+        <v>233</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>167</v>
+        <v>234</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>155</v>
+        <v>222</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="B83" s="7" t="n">
         <v>531.102863852944</v>
@@ -3180,7 +4132,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="s">
-        <v>94</v>
+        <v>161</v>
       </c>
       <c r="B85" s="10" t="n">
         <f aca="false">SUM(B83:B84)</f>
@@ -3193,21 +4145,21 @@
     </row>
     <row r="87" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="s">
-        <v>169</v>
+        <v>236</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>167</v>
+        <v>234</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>170</v>
+        <v>237</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>155</v>
+        <v>222</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>171</v>
+        <v>238</v>
       </c>
       <c r="B88" s="7" t="n">
         <v>221.156488366715</v>
@@ -3222,7 +4174,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>172</v>
+        <v>239</v>
       </c>
       <c r="B89" s="7" t="n">
         <v>84.3864815491803</v>
@@ -3237,7 +4189,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>173</v>
+        <v>240</v>
       </c>
       <c r="B90" s="7" t="n">
         <v>74.038</v>
@@ -3252,7 +4204,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>174</v>
+        <v>241</v>
       </c>
       <c r="B91" s="7" t="n">
         <v>50.85</v>
@@ -3267,7 +4219,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>175</v>
+        <v>242</v>
       </c>
       <c r="B92" s="7" t="n">
         <v>40.85</v>
@@ -3282,7 +4234,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>176</v>
+        <v>243</v>
       </c>
       <c r="B93" s="7" t="n">
         <v>26.3338573770492</v>
@@ -3297,7 +4249,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>177</v>
+        <v>244</v>
       </c>
       <c r="B94" s="7" t="n">
         <v>9.57</v>
@@ -3312,7 +4264,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>178</v>
+        <v>245</v>
       </c>
       <c r="B95" s="7" t="n">
         <v>5.50803083</v>
@@ -3327,7 +4279,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>179</v>
+        <v>246</v>
       </c>
       <c r="B96" s="7" t="n">
         <v>5.2</v>
@@ -3342,7 +4294,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="B97" s="7" t="n">
         <v>5.06</v>
@@ -3357,7 +4309,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>181</v>
+        <v>248</v>
       </c>
       <c r="B98" s="7" t="n">
         <v>4</v>
@@ -3372,7 +4324,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>182</v>
+        <v>249</v>
       </c>
       <c r="B99" s="7" t="n">
         <v>2.05</v>
@@ -3387,7 +4339,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>183</v>
+        <v>250</v>
       </c>
       <c r="B100" s="7" t="n">
         <v>1.19000573</v>
@@ -3402,7 +4354,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
-        <v>184</v>
+        <v>251</v>
       </c>
       <c r="B101" s="7" t="n">
         <v>0.51</v>
@@ -3417,7 +4369,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="s">
-        <v>94</v>
+        <v>161</v>
       </c>
       <c r="B102" s="10" t="n">
         <f aca="false">SUM(B88:B101)</f>
@@ -3431,12 +4383,12 @@
     </row>
     <row r="103" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>185</v>
+        <v>252</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>186</v>
+        <v>253</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3444,26 +4396,26 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="s">
-        <v>187</v>
+        <v>254</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="5" t="s">
-        <v>188</v>
+        <v>255</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>189</v>
+        <v>256</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>167</v>
+        <v>234</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>190</v>
+        <v>257</v>
       </c>
       <c r="B108" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C108" s="7" t="n">
         <v>61.0599999999998</v>
@@ -3471,10 +4423,10 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
-        <v>191</v>
+        <v>258</v>
       </c>
       <c r="B109" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C109" s="7" t="n">
         <v>53.0435999999999</v>
@@ -3482,10 +4434,10 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>192</v>
+        <v>259</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C110" s="7" t="n">
         <v>50</v>
@@ -3493,10 +4445,10 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="3" t="s">
-        <v>193</v>
+        <v>260</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C111" s="7" t="n">
         <v>33.9</v>
@@ -3504,10 +4456,10 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>194</v>
+        <v>261</v>
       </c>
       <c r="B112" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C112" s="7" t="n">
         <v>33.236361</v>
@@ -3515,10 +4467,10 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="3" t="s">
-        <v>195</v>
+        <v>262</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C113" s="7" t="n">
         <v>25.3501545</v>
@@ -3526,10 +4478,10 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>196</v>
+        <v>263</v>
       </c>
       <c r="B114" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C114" s="7" t="n">
         <v>21.6000445</v>
@@ -3537,10 +4489,10 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="3" t="s">
-        <v>197</v>
+        <v>264</v>
       </c>
       <c r="B115" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C115" s="7" t="n">
         <v>20.15022926</v>
@@ -3548,10 +4500,10 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>198</v>
+        <v>265</v>
       </c>
       <c r="B116" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C116" s="7" t="n">
         <v>18</v>
@@ -3559,10 +4511,10 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="3" t="s">
-        <v>199</v>
+        <v>266</v>
       </c>
       <c r="B117" s="9" t="s">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="C117" s="7" t="n">
         <v>14.15895</v>

</xml_diff>

<commit_message>
Approvers' backup: supplementary DMP tables for updated business answer
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TjyVtBMeKRjjZMJmWM6RZp
</commit_message>
<xml_diff>
--- a/BU2027_вопросы_согласующих_база.xlsx
+++ b/BU2027_вопросы_согласующих_база.xlsx
@@ -9,7 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="1. Вознаграждения РА" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="2. DMP — ответ бизнеса" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="2. DMP — доп. таблицы" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Справка DMP (внутр.)" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="267">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="256">
   <si>
     <t xml:space="preserve">1. Вознаграждения рекламным агентствам (суперкомиссия, СК): 2026 vs 2027, млн руб. без НДС</t>
   </si>
@@ -240,13 +240,172 @@
     <t xml:space="preserve">2026: янв–авг — факт начислений (премии РА признаются по итогам периодов, помесячная динамика неравномерна); сен–дек — прогноз мастера августа. 2027 — 795 / 12.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. DMP + Online: разбивка по направлениям 2026 vs 2027 (данные бизнеса), млн руб. без НДС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Источник: ответ бизнеса (команда DMP). Итоги сверены с бюджетной моделью cons 16.10.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.1 Выручка, маржинальность и затраты на трафик по направлениям</t>
+    <t xml:space="preserve">2. DMP + Online: дополнительные таблицы к ответу бизнеса, млн руб. без НДС</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Исходные данные по направлениям — таблица бизнеса (в этом листе — в сером блоке внизу, только для расчёта). Факт 2026 — «Расшифровка» мастера, 8 мес.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.1 Деньги, остающиеся Магниту (выручка − закупка трафика): 476 → 600, что дало +124</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фактор</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Эффект</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржа 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">987 − 511</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Рост объёма действующих направлений (по марже 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пакеты, баннеры и OLV, новые площадки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Снижение маржинальности новых площадок (уход ТГ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">−8 п.п. на 290 млн</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Новые пакеты на широких сегментах</t>
+  </si>
+  <si>
+    <t xml:space="preserve">440 млн × 15%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржа 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 600 − 1 000</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Каждый фактор положителен, кроме новых площадок: широкие сегменты не «съедают» маржу, а добавляют +66 млн при меньшей маржинальности.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.2 Мост маржинальности 48% → 37,5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Шаг</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржинальность</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027 без широких сегментов</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Новые площадки 52% → 44%; структура</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2027 с широкими сегментами</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Новые пакеты 440 млн при марже 15%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~80% снижения маржинальности дают новые пакеты на широких сегментах; без них маржинальность 2027 — 46%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3 Отдача прироста выручки: сколько копеек с рубля остаётся Магниту</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Блок</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прирост выручки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прирост маржи</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маржа на 1 руб. прироста</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Действующие направления</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Онлайн на широких сегментах</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого DMP + Online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Среднее 20 коп. — за счёт новых пакетов; по действующим направлениям — 34 коп.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.4 Масштаб новых пакетов на широких сегментах в бюджете AdTech 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Значение</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля в выручке DMP + Online 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля в выручке AdTech 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gross Revenue 14 566</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля в приросте выручки AdTech 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прирост +4 243</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вклад в EBITDA AdTech 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка за вычетом закупки трафика; СК по DMP не закладывается</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.5 Поставщики, названные в ответе: текущий объём сотрудничества, факт 8М 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Поставщик</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Выручка AdTech, всего</t>
+  </si>
+  <si>
+    <t xml:space="preserve">в т.ч. DMP + Online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доля DMP + Online</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Procter &amp; Gamble</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mondelez</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PepsiCo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Итого три поставщика</t>
+  </si>
+  <si>
+    <t xml:space="preserve">16% выручки DMP + Online 8М 2026 (530,7)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Все источники бюджета DMP + Online в 2026 — поставщики (100% выручки 8М). PepsiCo в DMP в 2026 не размещался — новые пакеты расширяют работу с ним.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Исходные данные (таблица бизнеса) — для формул</t>
   </si>
   <si>
     <t xml:space="preserve">Направление</t>
@@ -255,204 +414,18 @@
     <t xml:space="preserve">Выручка 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Маржа 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Трафик 2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Выручка 2027</t>
   </si>
   <si>
-    <t xml:space="preserve">Маржа 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Трафик 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Δ выручки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Δ маржи, п.п.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Комментарий бизнеса</t>
-  </si>
-  <si>
     <t xml:space="preserve">Пакеты и Онлайн+ТВ</t>
   </si>
   <si>
-    <t xml:space="preserve">Маржинальность без изменений</t>
-  </si>
-  <si>
     <t xml:space="preserve">Баннеры и OLV</t>
   </si>
   <si>
-    <t xml:space="preserve">Рост маржинальности за счёт улучшения условий закупки (рост объёмов)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Новые площадки (SmartTV, Авито, МР)</t>
   </si>
   <si>
-    <t xml:space="preserve">Снижение маржинальности за счёт ухода ТГ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Онлайн на широких сегментах (новое)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Новые пакеты 2027 по запросу маркетинга и крупных поставщиков (Pepsi, P&amp;G, Mondelez)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого по направлениям</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого по модели (P&amp;L)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маржинальность 48% → 37,5%: −10,7 п.п.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Расхождение: направления − модель</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Выручка по направлениям не сходится с итогом: 2026 — на 24 млн меньше, 2027 — на 11 млн больше</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Формулировка «маржинальность снижается на 11%» — это 11 п.п. (48% → 37,5%), а не 11%. Предлагаем писать «на ~11 п.п.».</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.2 Мост маржинальности 2026 → 2027</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Шаг</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маржинальность</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маржинальность 2026 (модель)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">987 / 511</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027 без «онлайна на широких сегментах»</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Действующие направления: баннеры +1 п.п., новые площадки −6,5 п.п. (уход ТГ), изменение структуры</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027 с «онлайном на широких сегментах»</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Новые пакеты 440 млн с маржой 17,5%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итог 2027 по модели (с учётом расхождения разбивки)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сумма направлений бизнеса больше итога модели на 11 млн</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого изменение</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~70% снижения маржинальности (−7,7 из −10,8 п.п.) дают новые пакеты на широких сегментах; действующие направления дают −2,6 п.п., в основном новые площадки (уход ТГ).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.3 Прирост выручки и денег, остающихся Магниту (к вопросу «20 копеек с рубля»)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Блок</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Прирост выручки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Прирост маржи (выручка − трафик)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маржа на 1 руб. прироста</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Действующие направления</t>
-  </si>
-  <si>
-    <t xml:space="preserve">По направлениям бизнеса (без расхождения с итогом модели)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Онлайн на широких сегментах</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого DMP+Online (модель)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">613 → +124: так считают согласующие</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.4 Сверка с бюджетной моделью: в модели другая разбивка по направлениям</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Направление в модели (лист DMP)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">В модели «широкие сегменты» не выделены: часть, видимо, внутри пакетов (маржа 25%)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого модель</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итоги модели и бизнеса совпадают (1 600 / 1 000 / 37,5%), разбивка — нет</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Закупка трафика в реестре: DMP+Online (ЦМ)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Отдельная строка реестра (ответственный — Ардаширов Д.). Похоже на «широкие сегменты по запросу маркетинга» (расход 363) — нужно подтвердить</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2.5 К тезису «все источники — поставщики, не РА; СК не выплачивается»</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Показатель, факт 8М 2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Значение</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Выручка DMP+Online, всего</t>
-  </si>
-  <si>
-    <t xml:space="preserve">«Расшифровка» мастера</t>
-  </si>
-  <si>
-    <t xml:space="preserve">в т.ч. от поставщиков</t>
-  </si>
-  <si>
-    <t xml:space="preserve">100% — подтверждает тезис бизнеса</t>
-  </si>
-  <si>
-    <t xml:space="preserve">в т.ч. проведено через РА (реальное направление «(РА)»)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">~29% выручки DMP+Online 8М шло через агентства</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Премии РА: data/online, начислено</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Небольшие премии РА по DMP в 2026 начислялись</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2027: DMP в базе СК</t>
-  </si>
-  <si>
-    <t xml:space="preserve">В расчёте СК 2027 база — не поставщики и бренд-бюджеты; DMP не входит</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Для 2026 тезис «не через РА, СК не выплачивается» фактом не подтверждается полностью. Безопаснее формулировка: «в бюджете 2027 СК по DMP не закладывается; бюджеты — поставщиков».</t>
-  </si>
-  <si>
     <t xml:space="preserve">2. DMP + Online: выручка, закупка трафика и маржинальность, млн руб. без НДС</t>
   </si>
   <si>
@@ -507,9 +480,6 @@
     <t xml:space="preserve">Комментария нет; в BU 2026 и факте 7М 2026 такой строки нет</t>
   </si>
   <si>
-    <t xml:space="preserve">Итого</t>
-  </si>
-  <si>
     <t xml:space="preserve">2.3 Маржинальность 2026: модель, P&amp;L 8+4 и реестр кампаний DMP</t>
   </si>
   <si>
@@ -709,9 +679,6 @@
   </si>
   <si>
     <t xml:space="preserve">МС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Итого DMP + Online</t>
   </si>
   <si>
     <t xml:space="preserve">В модели выручка DMP+Online разнесена на форматы по факту 8М 2026 (с корректировкой) — структура одинакова в обоих годах. Маржинальность по форматам в модели не считается (она задаётся по продуктам, п. 2.1).</t>
@@ -884,7 +851,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -894,13 +861,19 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
-        <bgColor rgb="FFC0C0C0"/>
+        <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFF2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -938,7 +911,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1015,19 +988,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1051,7 +1032,7 @@
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFF2F2F2"/>
       <rgbColor rgb="FFFF0000"/>
       <rgbColor rgb="FF00FF00"/>
       <rgbColor rgb="FF0000FF"/>
@@ -2039,35 +2020,28 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="50"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="J1" s="3"/>
-    </row>
-    <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="2" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="J3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="4" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>74</v>
       </c>
-      <c r="J4" s="3"/>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
@@ -2076,676 +2050,476 @@
       <c r="B5" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>84</v>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B6" s="17" t="n">
-        <v>220</v>
-      </c>
-      <c r="C6" s="8" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D6" s="17" t="n">
-        <f aca="false">IF(B6="","",B6*(1-C6))</f>
-        <v>132</v>
-      </c>
-      <c r="E6" s="17" t="n">
-        <v>292</v>
-      </c>
-      <c r="F6" s="8" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G6" s="17" t="n">
-        <f aca="false">E6*(1-F6)</f>
-        <v>175.2</v>
-      </c>
-      <c r="H6" s="17" t="n">
-        <f aca="false">E6-N(B6)</f>
-        <v>72</v>
-      </c>
-      <c r="I6" s="7" t="n">
-        <f aca="false">IF(C6="","",(F6-C6)*100)</f>
-        <v>0</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">SUM(B47:B50)-511</f>
+        <v>476</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="B7" s="17" t="n">
-        <v>505</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="D7" s="17" t="n">
-        <f aca="false">IF(B7="","",B7*(1-C7))</f>
-        <v>262.6</v>
-      </c>
-      <c r="E7" s="17" t="n">
-        <v>589</v>
-      </c>
-      <c r="F7" s="8" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="G7" s="17" t="n">
-        <f aca="false">E7*(1-F7)</f>
-        <v>300.39</v>
-      </c>
-      <c r="H7" s="17" t="n">
-        <f aca="false">E7-N(B7)</f>
-        <v>84</v>
-      </c>
-      <c r="I7" s="7" t="n">
-        <f aca="false">IF(C7="","",(F7-C7)*100)</f>
-        <v>1</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <f aca="false">(D47-B47)*C47+(D48-B48)*C48+(D49-B49)*C49</f>
+        <v>81.44</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="B8" s="17" t="n">
-        <v>238</v>
-      </c>
-      <c r="C8" s="8" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="D8" s="17" t="n">
-        <f aca="false">IF(B8="","",B8*(1-C8))</f>
-        <v>116.62</v>
-      </c>
-      <c r="E8" s="17" t="n">
-        <v>290</v>
-      </c>
-      <c r="F8" s="8" t="n">
-        <v>0.445</v>
-      </c>
-      <c r="G8" s="17" t="n">
-        <f aca="false">E8*(1-F8)</f>
-        <v>160.95</v>
-      </c>
-      <c r="H8" s="17" t="n">
-        <f aca="false">E8-N(B8)</f>
-        <v>52</v>
-      </c>
-      <c r="I8" s="7" t="n">
-        <f aca="false">IF(C8="","",(F8-C8)*100)</f>
-        <v>-6.5</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>90</v>
+        <f aca="false">D49*(E49-C49)</f>
+        <v>-23.2</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B9" s="17"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="17" t="str">
-        <f aca="false">IF(B9="","",B9*(1-C9))</f>
-        <v/>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>440</v>
-      </c>
-      <c r="F9" s="8" t="n">
-        <v>0.175</v>
-      </c>
-      <c r="G9" s="17" t="n">
-        <f aca="false">E9*(1-F9)</f>
-        <v>363</v>
-      </c>
-      <c r="H9" s="17" t="n">
-        <f aca="false">E9-N(B9)</f>
-        <v>440</v>
-      </c>
-      <c r="I9" s="7" t="str">
-        <f aca="false">IF(C9="","",(F9-C9)*100)</f>
-        <v/>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>92</v>
+        <v>83</v>
+      </c>
+      <c r="B9" s="17" t="n">
+        <f aca="false">D50*E50</f>
+        <v>66</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="18" t="n">
+        <f aca="false">B6+B7+B8+B9</f>
+        <v>600.24</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <f aca="false">(SUM(B47:B50)-511)/SUM(B47:B50)</f>
+        <v>0.482269503546099</v>
+      </c>
+      <c r="C15" s="7"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="8" t="n">
+        <f aca="false">(D47*E47+D48*E48+D49*E49)/(D47+D48+D49)</f>
+        <v>0.460775862068966</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <f aca="false">(B16-B15)*100</f>
+        <v>-2.14936414771337</v>
+      </c>
+      <c r="D16" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="18" t="n">
-        <f aca="false">SUM(B6:B9)</f>
-        <v>963</v>
-      </c>
-      <c r="C10" s="11" t="n">
-        <f aca="false">1-D10/B10</f>
-        <v>0.469138110072689</v>
-      </c>
-      <c r="D10" s="18" t="n">
-        <f aca="false">SUM(D6:D9)</f>
-        <v>511.22</v>
-      </c>
-      <c r="E10" s="18" t="n">
-        <f aca="false">SUM(E6:E9)</f>
-        <v>1611</v>
-      </c>
-      <c r="F10" s="11" t="n">
-        <f aca="false">1-G10/E10</f>
-        <v>0.379553072625698</v>
-      </c>
-      <c r="G10" s="18" t="n">
-        <f aca="false">SUM(G6:G9)</f>
-        <v>999.54</v>
-      </c>
-      <c r="H10" s="18" t="n">
-        <f aca="false">E10-B10</f>
-        <v>648</v>
-      </c>
-      <c r="I10" s="10" t="n">
-        <f aca="false">(F10-C10)*100</f>
-        <v>-8.95850374469911</v>
-      </c>
-      <c r="J10" s="3"/>
-    </row>
-    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B11" s="18" t="n">
-        <v>987</v>
-      </c>
-      <c r="C11" s="11" t="n">
-        <f aca="false">1-D11/B11</f>
-        <v>0.48273556231003</v>
-      </c>
-      <c r="D11" s="18" t="n">
-        <v>510.54</v>
-      </c>
-      <c r="E11" s="18" t="n">
-        <v>1600</v>
-      </c>
-      <c r="F11" s="11" t="n">
-        <f aca="false">1-G11/E11</f>
-        <v>0.375</v>
-      </c>
-      <c r="G11" s="18" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H11" s="18" t="n">
-        <f aca="false">E11-B11</f>
-        <v>613</v>
-      </c>
-      <c r="I11" s="10" t="n">
-        <f aca="false">(F11-C11)*100</f>
-        <v>-10.773556231003</v>
-      </c>
-      <c r="J11" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="B12" s="19" t="n">
-        <f aca="false">B10-B11</f>
-        <v>-24</v>
-      </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="20" t="n">
-        <f aca="false">D10-D11</f>
-        <v>0.680000000000007</v>
-      </c>
-      <c r="E12" s="19" t="n">
-        <f aca="false">E10-E11</f>
-        <v>11</v>
-      </c>
-      <c r="F12" s="15"/>
-      <c r="G12" s="20" t="n">
-        <f aca="false">G10-G11</f>
-        <v>-0.460000000000036</v>
-      </c>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="13" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="J13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3"/>
-      <c r="J14" s="3"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="J15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J16" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B17" s="8" t="n">
+        <f aca="false">(D47*E47+D48*E48+D49*E49+D50*E50)/SUM(D47:D50)</f>
+        <v>0.3753125</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <f aca="false">(B17-B16)*100</f>
+        <v>-8.54633620689656</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" s="12"/>
+      <c r="C18" s="10" t="n">
+        <f aca="false">(B17-B15)*100</f>
+        <v>-10.6957003546099</v>
+      </c>
+      <c r="D18" s="12"/>
+    </row>
+    <row r="19" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="2" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="B17" s="8" t="n">
-        <f aca="false">C11</f>
-        <v>0.48273556231003</v>
-      </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="3" t="s">
+      <c r="E22" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="J17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="3" t="s">
+      <c r="B23" s="17" t="n">
+        <f aca="false">(D47+D48+D49)-(B47+B48+B49)</f>
+        <v>173</v>
+      </c>
+      <c r="C23" s="17" t="n">
+        <f aca="false">(D47*E47+D48*E48+D49*E49)-(B47*C47+B48*C48+B49*C49)</f>
+        <v>58.24</v>
+      </c>
+      <c r="D23" s="19" t="n">
+        <f aca="false">C23/B23</f>
+        <v>0.336647398843931</v>
+      </c>
+      <c r="E23" s="3"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B18" s="8" t="n">
-        <f aca="false">1-SUM(G6:G8)/SUM(E6:E8)</f>
-        <v>0.456413321947054</v>
-      </c>
-      <c r="C18" s="7" t="n">
-        <f aca="false">(B18-B17)*100</f>
-        <v>-2.63222403629765</v>
-      </c>
-      <c r="D18" s="3" t="s">
+      <c r="B24" s="17" t="n">
+        <f aca="false">D50</f>
+        <v>440</v>
+      </c>
+      <c r="C24" s="17" t="n">
+        <f aca="false">D50*E50</f>
+        <v>66</v>
+      </c>
+      <c r="D24" s="19" t="n">
+        <f aca="false">C24/B24</f>
+        <v>0.15</v>
+      </c>
+      <c r="E24" s="3"/>
+    </row>
+    <row r="25" customFormat="false" ht="149.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="J18" s="3"/>
-    </row>
-    <row r="19" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="3" t="s">
+      <c r="B25" s="18" t="n">
+        <f aca="false">B23+B24</f>
+        <v>613</v>
+      </c>
+      <c r="C25" s="18" t="n">
+        <f aca="false">C23+C24</f>
+        <v>124.24</v>
+      </c>
+      <c r="D25" s="20" t="n">
+        <f aca="false">C25/B25</f>
+        <v>0.202675367047308</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="B19" s="8" t="n">
-        <f aca="false">F10</f>
-        <v>0.379553072625698</v>
-      </c>
-      <c r="C19" s="7" t="n">
-        <f aca="false">(B19-B18)*100</f>
-        <v>-7.68602493213555</v>
-      </c>
-      <c r="D19" s="3" t="s">
+    </row>
+    <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
         <v>107</v>
       </c>
-      <c r="J19" s="3"/>
-    </row>
-    <row r="20" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
+    </row>
+    <row r="28" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B28" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="B20" s="8" t="n">
-        <f aca="false">F11</f>
-        <v>0.375</v>
-      </c>
-      <c r="C20" s="7" t="n">
-        <f aca="false">(B20-B19)*100</f>
-        <v>-0.455307262569837</v>
-      </c>
-      <c r="D20" s="3" t="s">
+      <c r="C28" s="5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="J20" s="3"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="s">
+      <c r="B29" s="8" t="n">
+        <f aca="false">D50/SUM(D47:D50)</f>
+        <v>0.275</v>
+      </c>
+      <c r="C29" s="3"/>
+    </row>
+    <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B21" s="12"/>
-      <c r="C21" s="10" t="n">
-        <f aca="false">(B20-B17)*100</f>
-        <v>-10.773556231003</v>
-      </c>
-      <c r="D21" s="4"/>
-      <c r="J21" s="3"/>
-    </row>
-    <row r="22" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="B30" s="8" t="n">
+        <f aca="false">D50/14566.2</f>
+        <v>0.030206917384081</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="J22" s="3"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3"/>
-      <c r="J23" s="3"/>
-    </row>
-    <row r="24" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+    </row>
+    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="J24" s="3"/>
-    </row>
-    <row r="25" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="s">
+      <c r="B31" s="8" t="n">
+        <f aca="false">D50/4242.8</f>
+        <v>0.103705100405393</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B25" s="6" t="s">
+    </row>
+    <row r="32" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="B32" s="17" t="n">
+        <f aca="false">D50*E50</f>
+        <v>66</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D25" s="5" t="s">
+    </row>
+    <row r="34" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="E25" s="5" t="s">
+    </row>
+    <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E35" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="J25" s="3"/>
-    </row>
-    <row r="26" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="B26" s="17" t="n">
-        <f aca="false">SUM(E6:E8)-SUM(B6:B8)</f>
-        <v>208</v>
-      </c>
-      <c r="C26" s="17" t="n">
-        <f aca="false">(SUM(E6:E8)-SUM(G6:G8))-(SUM(B6:B8)-SUM(D6:D8))</f>
-        <v>82.6800000000001</v>
-      </c>
-      <c r="D26" s="21" t="n">
-        <f aca="false">C26/B26</f>
-        <v>0.3975</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="J26" s="3"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="B27" s="17" t="n">
-        <f aca="false">E9</f>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="B36" s="7" t="n">
+        <v>354.9</v>
+      </c>
+      <c r="C36" s="7" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="D36" s="8" t="n">
+        <f aca="false">C36/B36</f>
+        <v>0.0935474781628628</v>
+      </c>
+      <c r="E36" s="3"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B37" s="7" t="n">
+        <v>179.2</v>
+      </c>
+      <c r="C37" s="7" t="n">
+        <v>50</v>
+      </c>
+      <c r="D37" s="8" t="n">
+        <f aca="false">C37/B37</f>
+        <v>0.279017857142857</v>
+      </c>
+      <c r="E37" s="3"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B38" s="7" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="C38" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="8" t="n">
+        <f aca="false">C38/B38</f>
+        <v>0</v>
+      </c>
+      <c r="E38" s="3"/>
+    </row>
+    <row r="39" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B39" s="10" t="n">
+        <f aca="false">SUM(B36:B38)</f>
+        <v>580.6</v>
+      </c>
+      <c r="C39" s="10" t="n">
+        <f aca="false">SUM(C36:C38)</f>
+        <v>83.2</v>
+      </c>
+      <c r="D39" s="11" t="n">
+        <f aca="false">C39/B39</f>
+        <v>0.143300034447124</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B46" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D46" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="E46" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="B47" s="23" t="n">
+        <v>220</v>
+      </c>
+      <c r="C47" s="24" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D47" s="23" t="n">
+        <v>281</v>
+      </c>
+      <c r="E47" s="24" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="B48" s="23" t="n">
+        <v>529</v>
+      </c>
+      <c r="C48" s="24" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D48" s="23" t="n">
+        <v>589</v>
+      </c>
+      <c r="E48" s="24" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B49" s="23" t="n">
+        <v>238</v>
+      </c>
+      <c r="C49" s="24" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="D49" s="23" t="n">
+        <v>290</v>
+      </c>
+      <c r="E49" s="24" t="n">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="B50" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="23" t="n">
         <v>440</v>
       </c>
-      <c r="C27" s="17" t="n">
-        <f aca="false">E9-G9</f>
-        <v>77</v>
-      </c>
-      <c r="D27" s="21" t="n">
-        <f aca="false">C27/B27</f>
-        <v>0.175</v>
-      </c>
-      <c r="E27" s="3"/>
-      <c r="J27" s="3"/>
-    </row>
-    <row r="28" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
-        <v>120</v>
-      </c>
-      <c r="B28" s="18" t="n">
-        <f aca="false">E11-B11</f>
-        <v>613</v>
-      </c>
-      <c r="C28" s="18" t="n">
-        <f aca="false">(E11-G11)-(B11-D11)</f>
-        <v>123.54</v>
-      </c>
-      <c r="D28" s="22" t="n">
-        <f aca="false">C28/B28</f>
-        <v>0.201533442088091</v>
-      </c>
-      <c r="E28" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="J28" s="3"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3"/>
-      <c r="J29" s="3"/>
-    </row>
-    <row r="30" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="J30" s="3"/>
-    </row>
-    <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="E31" s="5"/>
-      <c r="F31" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="J31" s="3"/>
-    </row>
-    <row r="32" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B32" s="17" t="n">
-        <v>392.56</v>
-      </c>
-      <c r="C32" s="8" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D32" s="17" t="n">
-        <v>294.54</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="J32" s="3"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B33" s="17" t="n">
-        <v>787.91</v>
-      </c>
-      <c r="C33" s="8" t="n">
-        <v>0.404</v>
-      </c>
-      <c r="D33" s="17" t="n">
-        <v>469.38</v>
-      </c>
-      <c r="F33" s="3"/>
-      <c r="J33" s="3"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B34" s="17" t="n">
-        <v>419.53</v>
-      </c>
-      <c r="C34" s="8" t="n">
-        <v>0.437</v>
-      </c>
-      <c r="D34" s="17" t="n">
-        <v>236.08</v>
-      </c>
-      <c r="F34" s="3"/>
-      <c r="J34" s="3"/>
-    </row>
-    <row r="35" customFormat="false" ht="122.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B35" s="18" t="n">
-        <v>1600</v>
-      </c>
-      <c r="C35" s="11" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="D35" s="18" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E35" s="12"/>
-      <c r="F35" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="J35" s="3"/>
-    </row>
-    <row r="36" customFormat="false" ht="202.95" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="B36" s="19"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="19" t="n">
-        <v>404.45</v>
-      </c>
-      <c r="E36" s="15"/>
-      <c r="F36" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="J36" s="3"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="3"/>
-      <c r="J37" s="3"/>
-    </row>
-    <row r="38" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="J38" s="3"/>
-    </row>
-    <row r="39" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="J39" s="3"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>530.7</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>133</v>
-      </c>
-      <c r="J40" s="3"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B41" s="7" t="n">
-        <v>531.1</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="J41" s="3"/>
-    </row>
-    <row r="42" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="13" t="s">
-        <v>136</v>
-      </c>
-      <c r="B42" s="20" t="n">
-        <v>153.5</v>
-      </c>
-      <c r="C42" s="15" t="s">
-        <v>137</v>
-      </c>
-      <c r="J42" s="3"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="13" t="s">
-        <v>138</v>
-      </c>
-      <c r="B43" s="20" t="n">
-        <v>4.75</v>
-      </c>
-      <c r="C43" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="J43" s="3"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="B44" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>141</v>
-      </c>
-      <c r="J44" s="3"/>
-    </row>
-    <row r="45" customFormat="false" ht="82.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="J45" s="3"/>
+      <c r="E50" s="24" t="n">
+        <v>0.15</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2773,12 +2547,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2786,32 +2560,32 @@
     </row>
     <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>75</v>
+        <v>128</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>85</v>
+        <v>131</v>
       </c>
       <c r="B6" s="7" t="n">
         <v>392.559665831245</v>
@@ -2834,7 +2608,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>87</v>
+        <v>132</v>
       </c>
       <c r="B7" s="7" t="n">
         <v>787.912447786132</v>
@@ -2857,7 +2631,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="B8" s="7" t="n">
         <v>419.527886382623</v>
@@ -2880,7 +2654,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">SUM(B6:B8)</f>
@@ -2901,7 +2675,7 @@
     </row>
     <row r="10" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2909,45 +2683,45 @@
     </row>
     <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>156</v>
+        <v>147</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
       <c r="B14" s="7" t="n">
         <v>595.55</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>158</v>
+        <v>149</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="B15" s="7" t="n">
         <v>404.45</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>160</v>
+        <v>151</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>161</v>
+        <v>96</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>1000</v>
@@ -2959,24 +2733,24 @@
     </row>
     <row r="18" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>7</v>
@@ -2984,7 +2758,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="B20" s="7" t="n">
         <v>986.999999999999</v>
@@ -3001,12 +2775,12 @@
         <v>0.48273556231003</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="B21" s="7" t="n">
         <v>530.702863852945</v>
@@ -3023,12 +2797,12 @@
         <v>0.426260090157773</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B22" s="7" t="n">
         <v>530.702863852945</v>
@@ -3045,12 +2819,12 @@
         <v>0.198825854880224</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="B23" s="7" t="n">
         <v>369.316632851684</v>
@@ -3069,7 +2843,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>900.019496704628</v>
@@ -3086,12 +2860,12 @@
         <v>0.495857354200569</v>
       </c>
       <c r="F24" s="12" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="B25" s="7" t="n">
         <v>900.019496704628</v>
@@ -3110,7 +2884,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="B26" s="7" t="n">
         <v>546.94153</v>
@@ -3127,12 +2901,12 @@
         <v>0.658677998626936</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3140,7 +2914,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3189,7 +2963,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="B31" s="7" t="n">
         <v>16.9387687250432</v>
@@ -3234,7 +3008,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="B32" s="7" t="n">
         <v>28.52889409</v>
@@ -3279,7 +3053,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="B33" s="10" t="n">
         <f aca="false">B31-B32</f>
@@ -3336,7 +3110,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="B34" s="8" t="n">
         <f aca="false">IFERROR(B33/B31,"")</f>
@@ -3393,7 +3167,7 @@
     </row>
     <row r="35" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3401,15 +3175,15 @@
     </row>
     <row r="37" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>7</v>
@@ -3417,7 +3191,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="B39" s="7" t="n">
         <v>282.49799362</v>
@@ -3425,7 +3199,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="B40" s="7" t="n">
         <v>109.84879112</v>
@@ -3433,7 +3207,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="3" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="B41" s="7" t="n">
         <v>31.31843725</v>
@@ -3441,7 +3215,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="B42" s="7" t="n">
         <v>19.726605</v>
@@ -3449,7 +3223,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="B43" s="7" t="n">
         <v>16.0624436</v>
@@ -3457,7 +3231,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
       <c r="B44" s="7" t="n">
         <v>9.92231206</v>
@@ -3465,7 +3239,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="3" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="B45" s="7" t="n">
         <v>2.15214708</v>
@@ -3473,7 +3247,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="B46" s="7" t="n">
         <v>-46.34583669</v>
@@ -3481,7 +3255,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="3" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="B47" s="7" t="n">
         <v>-120.6984392</v>
@@ -3489,7 +3263,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="B48" s="10" t="n">
         <f aca="false">SUM(B39:B47)</f>
@@ -3502,35 +3276,35 @@
     </row>
     <row r="50" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="B52" s="7" t="n">
         <v>267.84</v>
@@ -3549,13 +3323,13 @@
         <f aca="false">IFERROR(1-E52/B52,"")</f>
         <v>0.639477572004224</v>
       </c>
-      <c r="G52" s="23" t="n">
+      <c r="G52" s="25" t="n">
         <v>75</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="3" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B53" s="7" t="n">
         <v>149.76153</v>
@@ -3574,13 +3348,13 @@
         <f aca="false">IFERROR(1-E53/B53,"")</f>
         <v>0.75765705792135</v>
       </c>
-      <c r="G53" s="23" t="n">
+      <c r="G53" s="25" t="n">
         <v>157</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="B54" s="7" t="n">
         <v>88</v>
@@ -3599,13 +3373,13 @@
         <f aca="false">IFERROR(1-E54/B54,"")</f>
         <v>0.487682909899352</v>
       </c>
-      <c r="G54" s="23" t="n">
+      <c r="G54" s="25" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="3" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="B55" s="7" t="n">
         <v>41.34</v>
@@ -3624,13 +3398,13 @@
         <f aca="false">IFERROR(1-E55/B55,"")</f>
         <v>0.788502737784228</v>
       </c>
-      <c r="G55" s="23" t="n">
+      <c r="G55" s="25" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>161</v>
+        <v>96</v>
       </c>
       <c r="B56" s="10" t="n">
         <f aca="false">SUM(B52:B55)</f>
@@ -3652,7 +3426,7 @@
         <f aca="false">IFERROR(1-E56/B56,"")</f>
         <v>0.658677998626936</v>
       </c>
-      <c r="G56" s="24" t="n">
+      <c r="G56" s="26" t="n">
         <f aca="false">SUM(G52:G55)</f>
         <v>280</v>
       </c>
@@ -3662,30 +3436,30 @@
     </row>
     <row r="58" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="D58" s="6" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="3" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="B59" s="7" t="n">
         <v>130.8826</v>
@@ -3704,13 +3478,13 @@
         <f aca="false">IFERROR(1-E59/B59,"")</f>
         <v>0.725782153089869</v>
       </c>
-      <c r="G59" s="23" t="n">
+      <c r="G59" s="25" t="n">
         <v>134</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="B60" s="7" t="n">
         <v>117.71</v>
@@ -3729,13 +3503,13 @@
         <f aca="false">IFERROR(1-E60/B60,"")</f>
         <v>0.752562215067636</v>
       </c>
-      <c r="G60" s="23" t="n">
+      <c r="G60" s="25" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="3" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="B61" s="7" t="n">
         <v>88</v>
@@ -3754,13 +3528,13 @@
         <f aca="false">IFERROR(1-E61/B61,"")</f>
         <v>0.487682909899352</v>
       </c>
-      <c r="G61" s="23" t="n">
+      <c r="G61" s="25" t="n">
         <v>23</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="B62" s="7" t="n">
         <v>72.5556</v>
@@ -3779,13 +3553,13 @@
         <f aca="false">IFERROR(1-E62/B62,"")</f>
         <v>0.612268256206275</v>
       </c>
-      <c r="G62" s="23" t="n">
+      <c r="G62" s="25" t="n">
         <v>50</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="3" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="B63" s="7" t="n">
         <v>50</v>
@@ -3804,13 +3578,13 @@
         <f aca="false">IFERROR(1-E63/B63,"")</f>
         <v>0.4466189338</v>
       </c>
-      <c r="G63" s="23" t="n">
+      <c r="G63" s="25" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="B64" s="7" t="n">
         <v>41.34</v>
@@ -3829,13 +3603,13 @@
         <f aca="false">IFERROR(1-E64/B64,"")</f>
         <v>0.788502737784228</v>
       </c>
-      <c r="G64" s="23" t="n">
+      <c r="G64" s="25" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="B65" s="7" t="n">
         <v>23.50433</v>
@@ -3854,13 +3628,13 @@
         <f aca="false">IFERROR(1-E65/B65,"")</f>
         <v>0.589605352698843</v>
       </c>
-      <c r="G65" s="23" t="n">
+      <c r="G65" s="25" t="n">
         <v>16</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="B66" s="7" t="n">
         <v>12.359</v>
@@ -3879,13 +3653,13 @@
         <f aca="false">IFERROR(1-E66/B66,"")</f>
         <v>0.999979091350433</v>
       </c>
-      <c r="G66" s="23" t="n">
+      <c r="G66" s="25" t="n">
         <v>11</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="B67" s="7" t="n">
         <v>6</v>
@@ -3904,13 +3678,13 @@
         <f aca="false">IFERROR(1-E67/B67,"")</f>
         <v>0.6013</v>
       </c>
-      <c r="G67" s="23" t="n">
+      <c r="G67" s="25" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="B68" s="7" t="n">
         <v>4.59</v>
@@ -3929,13 +3703,13 @@
         <f aca="false">IFERROR(1-E68/B68,"")</f>
         <v>0.99998731590414</v>
       </c>
-      <c r="G68" s="23" t="n">
+      <c r="G68" s="25" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="2" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3943,32 +3717,32 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="4" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="5" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="D72" s="6" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="B73" s="7" t="n">
         <v>768.821180909195</v>
@@ -3991,7 +3765,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="B74" s="7" t="n">
         <v>192.791639187493</v>
@@ -4014,7 +3788,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="B75" s="7" t="n">
         <v>18.942306944518</v>
@@ -4037,7 +3811,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="B76" s="7" t="n">
         <v>6.44487295879252</v>
@@ -4060,7 +3834,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>229</v>
+        <v>105</v>
       </c>
       <c r="B77" s="10" t="n">
         <f aca="false">SUM(B73:B76)</f>
@@ -4079,12 +3853,12 @@
     </row>
     <row r="78" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="2" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="2" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4092,23 +3866,23 @@
     </row>
     <row r="81" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="5" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="C82" s="6" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="B83" s="7" t="n">
         <v>531.102863852944</v>
@@ -4132,7 +3906,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="s">
-        <v>161</v>
+        <v>96</v>
       </c>
       <c r="B85" s="10" t="n">
         <f aca="false">SUM(B83:B84)</f>
@@ -4145,21 +3919,21 @@
     </row>
     <row r="87" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="5" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="D87" s="6" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="B88" s="7" t="n">
         <v>221.156488366715</v>
@@ -4174,7 +3948,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="B89" s="7" t="n">
         <v>84.3864815491803</v>
@@ -4189,7 +3963,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="B90" s="7" t="n">
         <v>74.038</v>
@@ -4204,7 +3978,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="B91" s="7" t="n">
         <v>50.85</v>
@@ -4219,7 +3993,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="B92" s="7" t="n">
         <v>40.85</v>
@@ -4234,7 +4008,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="B93" s="7" t="n">
         <v>26.3338573770492</v>
@@ -4249,7 +4023,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="B94" s="7" t="n">
         <v>9.57</v>
@@ -4264,7 +4038,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="B95" s="7" t="n">
         <v>5.50803083</v>
@@ -4279,7 +4053,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>246</v>
+        <v>235</v>
       </c>
       <c r="B96" s="7" t="n">
         <v>5.2</v>
@@ -4294,7 +4068,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="B97" s="7" t="n">
         <v>5.06</v>
@@ -4309,7 +4083,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="B98" s="7" t="n">
         <v>4</v>
@@ -4324,7 +4098,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="B99" s="7" t="n">
         <v>2.05</v>
@@ -4339,7 +4113,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="B100" s="7" t="n">
         <v>1.19000573</v>
@@ -4354,7 +4128,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="B101" s="7" t="n">
         <v>0.51</v>
@@ -4369,7 +4143,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="4" t="s">
-        <v>161</v>
+        <v>96</v>
       </c>
       <c r="B102" s="10" t="n">
         <f aca="false">SUM(B88:B101)</f>
@@ -4383,12 +4157,12 @@
     </row>
     <row r="103" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="2" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4396,26 +4170,26 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="4" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="5" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="B108" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C108" s="7" t="n">
         <v>61.0599999999998</v>
@@ -4423,10 +4197,10 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="B109" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C109" s="7" t="n">
         <v>53.0435999999999</v>
@@ -4434,10 +4208,10 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C110" s="7" t="n">
         <v>50</v>
@@ -4445,10 +4219,10 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="3" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C111" s="7" t="n">
         <v>33.9</v>
@@ -4456,10 +4230,10 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="B112" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C112" s="7" t="n">
         <v>33.236361</v>
@@ -4467,10 +4241,10 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="3" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C113" s="7" t="n">
         <v>25.3501545</v>
@@ -4478,10 +4252,10 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="B114" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C114" s="7" t="n">
         <v>21.6000445</v>
@@ -4489,10 +4263,10 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="3" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="B115" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C115" s="7" t="n">
         <v>20.15022926</v>
@@ -4500,10 +4274,10 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="B116" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C116" s="7" t="n">
         <v>18</v>
@@ -4511,10 +4285,10 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="3" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="B117" s="9" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C117" s="7" t="n">
         <v>14.15895</v>

</xml_diff>